<commit_message>
return updated to end of 2024
</commit_message>
<xml_diff>
--- a/static/returns/returns.xlsx
+++ b/static/returns/returns.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work Files\ips generator\ips_generator\static\returns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C339E80D-A81C-46B3-828E-1B18D9F9D533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C75FC7-26DA-430C-90EF-0917827AD1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{3B7D21DE-0BB4-48EB-8D25-721726C207C8}"/>
+    <workbookView xWindow="2865" yWindow="3405" windowWidth="38700" windowHeight="15345" xr2:uid="{3B7D21DE-0BB4-48EB-8D25-721726C207C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -110,9 +110,6 @@
     <t>2018b</t>
   </si>
   <si>
-    <t>2017b</t>
-  </si>
-  <si>
     <t>Beutel Goodman Conservative Balanced</t>
   </si>
   <si>
@@ -257,10 +254,13 @@
     <t>2018a</t>
   </si>
   <si>
-    <t>2017a</t>
-  </si>
-  <si>
     <t>Hamilton Lane Global Private Assets Fund</t>
+  </si>
+  <si>
+    <t>2024a</t>
+  </si>
+  <si>
+    <t>2024b</t>
   </si>
 </sst>
 </file>
@@ -312,10 +312,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -714,2594 +715,2594 @@
         <v>17</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="X1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="Z1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" t="s">
-        <v>26</v>
-      </c>
       <c r="C2" s="2">
-        <v>1.9380146341463341E-2</v>
+        <v>-1.52E-2</v>
       </c>
       <c r="D2" s="2">
-        <v>6.6356448991957695E-2</v>
+        <v>-4.4000000000000003E-3</v>
       </c>
       <c r="E2" s="2">
-        <v>7.5854482362777809E-2</v>
+        <v>7.1099999999999997E-2</v>
       </c>
       <c r="F2" s="2">
-        <v>0.16550915215889961</v>
+        <v>7.1099999999999997E-2</v>
       </c>
       <c r="G2" s="2">
-        <v>3.5847941311260463E-2</v>
+        <v>2.23E-2</v>
       </c>
       <c r="H2" s="2">
-        <v>4.9090544625267851E-2</v>
+        <v>4.7899999999999998E-2</v>
       </c>
       <c r="I2" s="2">
-        <v>4.844840816613849E-2</v>
+        <v>4.6699999999999998E-2</v>
       </c>
       <c r="J2" s="2">
-        <v>6.0413183617088917E-2</v>
+        <v>5.9499999999999997E-2</v>
       </c>
       <c r="K2" s="2">
-        <v>2.2200000000000001E-2</v>
+        <v>-1.2E-2</v>
       </c>
       <c r="L2" s="2">
-        <v>5.9671296499999922E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="M2" s="2">
-        <v>8.5932057496088676E-2</v>
+        <v>0.1022</v>
       </c>
       <c r="N2" s="2">
-        <v>0.17265677007298769</v>
+        <v>0.1022</v>
       </c>
       <c r="O2" s="2">
-        <v>3.137281212711085E-2</v>
+        <v>2.5399999999999999E-2</v>
       </c>
       <c r="P2" s="2">
-        <v>4.2551197990956517E-2</v>
+        <v>4.4299999999999999E-2</v>
       </c>
       <c r="Q2" s="2">
-        <v>4.5323690024229528E-2</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="R2" s="2">
-        <v>5.3855256695795939E-2</v>
+        <v>5.3900000000000003E-2</v>
       </c>
       <c r="S2" s="2">
-        <v>6.9503962505472972E-2</v>
+        <v>7.1099999999999997E-2</v>
       </c>
       <c r="T2" s="2">
-        <v>-6.7351246961500744E-2</v>
+        <v>6.9500000000000006E-2</v>
       </c>
       <c r="U2" s="2">
-        <v>8.5023922266367569E-2</v>
+        <v>-6.7400000000000002E-2</v>
       </c>
       <c r="V2" s="2">
-        <v>8.9842946766752751E-2</v>
+        <v>8.5000000000000006E-2</v>
       </c>
       <c r="W2" s="2">
-        <v>0.10176585775880009</v>
+        <v>8.9800000000000005E-2</v>
       </c>
       <c r="X2" s="2">
-        <v>-2.6719568605251261E-3</v>
+        <v>0.1018</v>
       </c>
       <c r="Y2" s="2">
-        <v>4.4222136762895659E-2</v>
+        <v>-2.7000000000000001E-3</v>
       </c>
       <c r="Z2" s="2">
-        <v>8.7716228179286926E-2</v>
+        <v>0.1022</v>
       </c>
       <c r="AA2" s="2">
-        <v>-0.1007791321090222</v>
+        <v>8.77E-2</v>
       </c>
       <c r="AB2" s="2">
-        <v>5.4533862712955017E-2</v>
+        <v>-0.1008</v>
       </c>
       <c r="AC2" s="2">
-        <v>9.2753957970583167E-2</v>
+        <v>5.45E-2</v>
       </c>
       <c r="AD2" s="2">
-        <v>0.1168755683777853</v>
+        <v>9.2799999999999994E-2</v>
       </c>
       <c r="AE2" s="2">
-        <v>-3.3133518868777578E-4</v>
+        <v>0.1169</v>
       </c>
       <c r="AF2" s="2">
-        <v>4.8316637829175717E-2</v>
+        <v>-2.9999999999999997E-4</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" t="s">
-        <v>28</v>
-      </c>
       <c r="C3" s="2">
-        <v>1.5855625850340171E-2</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="D3" s="2">
-        <v>4.1970346605364028E-2</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="E3" s="2">
-        <v>4.896866141174927E-2</v>
+        <v>5.1700000000000003E-2</v>
       </c>
       <c r="F3" s="2">
-        <v>0.1141860497799634</v>
+        <v>5.1700000000000003E-2</v>
       </c>
       <c r="G3" s="2">
-        <v>8.3914603797787812E-3</v>
+        <v>1.04E-2</v>
       </c>
       <c r="H3" s="2">
-        <v>1.4909245670584379E-2</v>
+        <v>1.6199999999999999E-2</v>
       </c>
       <c r="I3" s="2">
-        <v>1.975645032982332E-2</v>
+        <v>1.9099999999999999E-2</v>
       </c>
       <c r="J3" s="2">
-        <v>4.4067559116196968E-2</v>
+        <v>4.3799999999999999E-2</v>
       </c>
       <c r="K3" s="2">
-        <v>1.5500000000000069E-2</v>
+        <v>1.5E-3</v>
       </c>
       <c r="L3" s="2">
-        <v>4.0990563095000272E-2</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="M3" s="2">
-        <v>5.0628411126180987E-2</v>
+        <v>5.3400000000000003E-2</v>
       </c>
       <c r="N3" s="2">
-        <v>0.10891234531006749</v>
+        <v>5.3400000000000003E-2</v>
       </c>
       <c r="O3" s="2">
-        <v>1.201530251901217E-2</v>
+        <v>1.3599999999999999E-2</v>
       </c>
       <c r="P3" s="2">
-        <v>1.590953574670095E-2</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="Q3" s="2">
-        <v>2.0723843198017899E-2</v>
+        <v>1.9400000000000001E-2</v>
       </c>
       <c r="R3" s="2">
-        <v>4.1415242505372429E-2</v>
+        <v>4.1099999999999998E-2</v>
       </c>
       <c r="S3" s="2">
-        <v>5.9227296447104998E-2</v>
+        <v>5.1700000000000003E-2</v>
       </c>
       <c r="T3" s="2">
-        <v>-7.4084527114463228E-2</v>
+        <v>5.9200000000000003E-2</v>
       </c>
       <c r="U3" s="2">
-        <v>-2.07639840561471E-2</v>
+        <v>-7.4099999999999999E-2</v>
       </c>
       <c r="V3" s="2">
-        <v>7.2733709335903507E-2</v>
+        <v>-2.0799999999999999E-2</v>
       </c>
       <c r="W3" s="2">
-        <v>4.2417853556049989E-2</v>
+        <v>7.2700000000000001E-2</v>
       </c>
       <c r="X3" s="2">
-        <v>1.5143026145177931E-2</v>
+        <v>4.24E-2</v>
       </c>
       <c r="Y3" s="2">
-        <v>6.3711307304896714E-3</v>
+        <v>1.5100000000000001E-2</v>
       </c>
       <c r="Z3" s="2">
-        <v>5.4237633096663178E-2</v>
+        <v>5.3400000000000003E-2</v>
       </c>
       <c r="AA3" s="2">
-        <v>-6.2297397020487977E-2</v>
+        <v>5.4199999999999998E-2</v>
       </c>
       <c r="AB3" s="2">
-        <v>-1.533915638406891E-2</v>
+        <v>-6.2300000000000001E-2</v>
       </c>
       <c r="AC3" s="2">
-        <v>6.1174539832829611E-2</v>
+        <v>-1.5299999999999999E-2</v>
       </c>
       <c r="AD3" s="2">
-        <v>4.0268031248332781E-2</v>
+        <v>6.1199999999999997E-2</v>
       </c>
       <c r="AE3" s="2">
-        <v>1.9121810314036921E-2</v>
+        <v>4.0300000000000002E-2</v>
       </c>
       <c r="AF3" s="2">
-        <v>3.8914714728139899E-3</v>
+        <v>1.9099999999999999E-2</v>
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
         <v>29</v>
       </c>
-      <c r="B4" t="s">
-        <v>30</v>
-      </c>
       <c r="C4" s="2">
-        <v>1.2634843049327269E-2</v>
+        <v>-1.6899999999999998E-2</v>
       </c>
       <c r="D4" s="2">
-        <v>6.0046530427247717E-2</v>
+        <v>3.73E-2</v>
       </c>
       <c r="E4" s="2">
-        <v>0.15975502016774309</v>
+        <v>0.20300000000000001</v>
       </c>
       <c r="F4" s="2">
-        <v>0.27007233787570589</v>
+        <v>0.20300000000000001</v>
       </c>
       <c r="G4" s="2">
-        <v>0.14569793188944449</v>
+        <v>0.12570000000000001</v>
       </c>
       <c r="H4" s="2">
-        <v>0.15616937649944809</v>
+        <v>0.15709999999999999</v>
       </c>
       <c r="I4" s="2">
-        <v>0.1291847550940517</v>
+        <v>0.12970000000000001</v>
       </c>
       <c r="J4" s="2">
-        <v>9.8680593706173658E-2</v>
+        <v>9.9299999999999999E-2</v>
       </c>
       <c r="K4" s="2">
-        <v>2.849999999999997E-2</v>
+        <v>-2.2700000000000001E-2</v>
       </c>
       <c r="L4" s="2">
-        <v>9.1615908075000085E-2</v>
+        <v>5.3600000000000002E-2</v>
       </c>
       <c r="M4" s="2">
-        <v>0.19201987377505339</v>
+        <v>0.25590000000000002</v>
       </c>
       <c r="N4" s="2">
-        <v>0.29164091098966999</v>
+        <v>0.25590000000000002</v>
       </c>
       <c r="O4" s="2">
-        <v>0.11260537685346921</v>
+        <v>0.1013</v>
       </c>
       <c r="P4" s="2">
-        <v>0.1282660010542018</v>
+        <v>0.13170000000000001</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.1077118786296689</v>
+        <v>0.1109</v>
       </c>
       <c r="R4" s="2">
-        <v>6.6800013440742267E-2</v>
+        <v>6.8400000000000002E-2</v>
       </c>
       <c r="S4" s="2">
-        <v>0.22666917874780079</v>
+        <v>0.20300000000000001</v>
       </c>
       <c r="T4" s="2">
-        <v>-3.3374670046121817E-2</v>
+        <v>0.22670000000000001</v>
       </c>
       <c r="U4" s="2">
-        <v>0.29477003772115862</v>
+        <v>-3.3399999999999999E-2</v>
       </c>
       <c r="V4" s="2">
-        <v>0.12321388075036779</v>
+        <v>0.29480000000000001</v>
       </c>
       <c r="W4" s="2">
-        <v>0.1946031324946251</v>
+        <v>0.1232</v>
       </c>
       <c r="X4" s="2">
-        <v>-2.283559756047659E-3</v>
+        <v>0.1946</v>
       </c>
       <c r="Y4" s="2">
-        <v>0.12426331877865079</v>
+        <v>-2.3E-3</v>
       </c>
       <c r="Z4" s="2">
-        <v>0.1488587438947935</v>
+        <v>0.25590000000000002</v>
       </c>
       <c r="AA4" s="2">
-        <v>-7.4243142523677252E-2</v>
+        <v>0.1489</v>
       </c>
       <c r="AB4" s="2">
-        <v>0.27962037205920343</v>
+        <v>-7.4200000000000002E-2</v>
       </c>
       <c r="AC4" s="2">
-        <v>8.6160849121817984E-2</v>
+        <v>0.27960000000000002</v>
       </c>
       <c r="AD4" s="2">
-        <v>0.22822661859954649</v>
+        <v>8.6199999999999999E-2</v>
       </c>
       <c r="AE4" s="2">
-        <v>-4.0965727438507897E-2</v>
+        <v>0.22819999999999999</v>
       </c>
       <c r="AF4" s="2">
-        <v>0.1101306155396751</v>
+        <v>-4.1000000000000002E-2</v>
       </c>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
         <v>31</v>
       </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
       <c r="C5" s="2">
-        <v>2.4559951219512269E-2</v>
+        <v>-1.6E-2</v>
       </c>
       <c r="D5" s="2">
-        <v>8.3689304932301534E-2</v>
+        <v>2.3099999999999999E-2</v>
       </c>
       <c r="E5" s="2">
-        <v>0.14264153628665621</v>
+        <v>0.1691</v>
       </c>
       <c r="F5" s="2">
-        <v>0.24246551527303881</v>
+        <v>0.1691</v>
       </c>
       <c r="G5" s="2">
-        <v>7.7301978031459884E-2</v>
+        <v>6.7900000000000002E-2</v>
       </c>
       <c r="H5" s="2">
-        <v>7.7443058488650962E-2</v>
+        <v>8.1299999999999997E-2</v>
       </c>
       <c r="I5" s="2">
-        <v>6.5375631746704466E-2</v>
+        <v>6.7299999999999999E-2</v>
       </c>
       <c r="J5" s="2">
-        <v>7.7055677944409373E-2</v>
+        <v>7.7200000000000005E-2</v>
       </c>
       <c r="K5" s="2">
-        <v>2.6499999999999971E-2</v>
+        <v>-2.24E-2</v>
       </c>
       <c r="L5" s="2">
-        <v>8.1607057129999827E-2</v>
+        <v>2.2599999999999999E-2</v>
       </c>
       <c r="M5" s="2">
-        <v>0.1190494106059181</v>
+        <v>0.1444</v>
       </c>
       <c r="N5" s="2">
-        <v>0.20905347096464449</v>
+        <v>0.1444</v>
       </c>
       <c r="O5" s="2">
-        <v>5.7533940213279511E-2</v>
+        <v>0.05</v>
       </c>
       <c r="P5" s="2">
-        <v>7.0791563533335822E-2</v>
+        <v>7.2300000000000003E-2</v>
       </c>
       <c r="Q5" s="2">
-        <v>5.9707680756499133E-2</v>
+        <v>6.1899999999999997E-2</v>
       </c>
       <c r="R5" s="2">
-        <v>7.3961874483091217E-2</v>
+        <v>7.4099999999999999E-2</v>
       </c>
       <c r="S5" s="2">
-        <v>0.12328855877582499</v>
+        <v>0.1691</v>
       </c>
       <c r="T5" s="2">
-        <v>-7.2623009670554461E-2</v>
+        <v>0.12330000000000001</v>
       </c>
       <c r="U5" s="2">
-        <v>0.13359880186010689</v>
+        <v>-7.2599999999999998E-2</v>
       </c>
       <c r="V5" s="2">
-        <v>7.0964251198278427E-2</v>
+        <v>0.1336</v>
       </c>
       <c r="W5" s="2">
-        <v>0.1324110955443196</v>
+        <v>7.0999999999999994E-2</v>
       </c>
       <c r="X5" s="2">
-        <v>-2.7766693482052299E-2</v>
+        <v>0.13239999999999999</v>
       </c>
       <c r="Y5" s="2">
-        <v>7.7382244985983339E-2</v>
+        <v>-2.7799999999999998E-2</v>
       </c>
       <c r="Z5" s="2">
-        <v>9.7290450620474145E-2</v>
+        <v>0.1444</v>
       </c>
       <c r="AA5" s="2">
-        <v>-7.8060196500178036E-2</v>
+        <v>9.7299999999999998E-2</v>
       </c>
       <c r="AB5" s="2">
-        <v>0.1351871011014274</v>
+        <v>-7.8100000000000003E-2</v>
       </c>
       <c r="AC5" s="2">
-        <v>7.8614809902556315E-2</v>
+        <v>0.13519999999999999</v>
       </c>
       <c r="AD5" s="2">
-        <v>0.16333273441343341</v>
+        <v>7.8600000000000003E-2</v>
       </c>
       <c r="AE5" s="2">
-        <v>-4.6556803672422993E-2</v>
+        <v>0.1633</v>
       </c>
       <c r="AF5" s="2">
-        <v>6.4707613131943065E-2</v>
+        <v>-4.6600000000000003E-2</v>
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" t="s">
-        <v>34</v>
-      </c>
       <c r="C6" s="2">
-        <v>2.7758600000000081E-2</v>
+        <v>-2.1600000000000001E-2</v>
       </c>
       <c r="D6" s="2">
-        <v>0.1042063541205689</v>
+        <v>3.7900000000000003E-2</v>
       </c>
       <c r="E6" s="2">
-        <v>0.20094751159993601</v>
+        <v>0.2465</v>
       </c>
       <c r="F6" s="2">
-        <v>0.3063722122544732</v>
+        <v>0.2465</v>
       </c>
       <c r="G6" s="2">
-        <v>0.12224401242238001</v>
+        <v>0.1099</v>
       </c>
       <c r="H6" s="2">
-        <v>0.11106612926658729</v>
+        <v>0.11650000000000001</v>
       </c>
       <c r="I6" s="2">
-        <v>8.5143453374761258E-2</v>
+        <v>9.0200000000000002E-2</v>
       </c>
       <c r="J6" s="2">
-        <v>8.430023582191537E-2</v>
+        <v>8.5000000000000006E-2</v>
       </c>
       <c r="K6" s="2">
-        <v>3.1500000000000077E-2</v>
+        <v>-3.27E-2</v>
       </c>
       <c r="L6" s="2">
-        <v>0.10537204841</v>
+        <v>3.7699999999999997E-2</v>
       </c>
       <c r="M6" s="2">
-        <v>0.1722477759505909</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="N6" s="2">
-        <v>0.27034955217191731</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="O6" s="2">
-        <v>9.59203442098151E-2</v>
+        <v>8.6499999999999994E-2</v>
       </c>
       <c r="P6" s="2">
-        <v>0.1099255546061737</v>
+        <v>0.11119999999999999</v>
       </c>
       <c r="Q6" s="2">
-        <v>8.1103140812044172E-2</v>
+        <v>8.6699999999999999E-2</v>
       </c>
       <c r="R6" s="2">
-        <v>7.3864750916512012E-2</v>
+        <v>7.46E-2</v>
       </c>
       <c r="S6" s="2">
-        <v>0.1481932347269663</v>
+        <v>0.2465</v>
       </c>
       <c r="T6" s="2">
-        <v>-4.4647519966674272E-2</v>
+        <v>0.1482</v>
       </c>
       <c r="U6" s="2">
-        <v>0.22858982038478379</v>
+        <v>-4.4600000000000001E-2</v>
       </c>
       <c r="V6" s="2">
-        <v>3.2613190352135168E-2</v>
+        <v>0.2286</v>
       </c>
       <c r="W6" s="2">
-        <v>0.16910836648109909</v>
+        <v>3.2599999999999997E-2</v>
       </c>
       <c r="X6" s="2">
-        <v>-6.0702708212991729E-2</v>
+        <v>0.1691</v>
       </c>
       <c r="Y6" s="2">
-        <v>0.1075353222141979</v>
+        <v>-6.0699999999999997E-2</v>
       </c>
       <c r="Z6" s="2">
-        <v>0.12021853546487481</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="AA6" s="2">
-        <v>-5.861422986020437E-2</v>
+        <v>0.1202</v>
       </c>
       <c r="AB6" s="2">
-        <v>0.25087973789207202</v>
+        <v>-5.8599999999999999E-2</v>
       </c>
       <c r="AC6" s="2">
-        <v>5.5915166451887321E-2</v>
+        <v>0.25090000000000001</v>
       </c>
       <c r="AD6" s="2">
-        <v>0.22876839007651761</v>
+        <v>5.5899999999999998E-2</v>
       </c>
       <c r="AE6" s="2">
-        <v>-8.8861093780151279E-2</v>
+        <v>0.2288</v>
       </c>
       <c r="AF6" s="2">
-        <v>9.0951444205845222E-2</v>
+        <v>-8.8900000000000007E-2</v>
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" t="s">
         <v>35</v>
       </c>
-      <c r="B7" t="s">
-        <v>36</v>
-      </c>
       <c r="C7" s="2">
-        <v>2.070125210084028E-2</v>
+        <v>-6.4000000000000003E-3</v>
       </c>
       <c r="D7" s="2">
-        <v>5.0883307898063057E-2</v>
+        <v>1E-4</v>
       </c>
       <c r="E7" s="2">
-        <v>4.9619589200431642E-2</v>
+        <v>4.9799999999999997E-2</v>
       </c>
       <c r="F7" s="2">
-        <v>0.14334619384045369</v>
+        <v>4.9799999999999997E-2</v>
       </c>
       <c r="G7" s="2">
-        <v>1.556416393702964E-3</v>
+        <v>-4.3E-3</v>
       </c>
       <c r="H7" s="2">
-        <v>9.8136928190490913E-3</v>
+        <v>1.2E-2</v>
       </c>
       <c r="I7" s="2">
-        <v>2.3498731255301001E-2</v>
+        <v>2.1100000000000001E-2</v>
       </c>
       <c r="J7" s="2">
-        <v>5.2607452630164531E-2</v>
+        <v>5.2200000000000003E-2</v>
       </c>
       <c r="K7" s="2">
-        <v>1.9099999999999891E-2</v>
+        <v>-6.8999999999999999E-3</v>
       </c>
       <c r="L7" s="2">
-        <v>4.659107854400002E-2</v>
+        <v>-5.0000000000000001E-4</v>
       </c>
       <c r="M7" s="2">
-        <v>4.2794816038896011E-2</v>
+        <v>4.2299999999999997E-2</v>
       </c>
       <c r="N7" s="2">
-        <v>0.124976108740396</v>
+        <v>4.2299999999999997E-2</v>
       </c>
       <c r="O7" s="2">
-        <v>-2.2046397650784528E-3</v>
+        <v>-7.1999999999999998E-3</v>
       </c>
       <c r="P7" s="2">
-        <v>5.5507327550163854E-3</v>
+        <v>7.1999999999999998E-3</v>
       </c>
       <c r="Q7" s="2">
-        <v>2.2170375268985461E-2</v>
+        <v>1.9400000000000001E-2</v>
       </c>
       <c r="R7" s="2">
-        <v>5.1070507372025453E-2</v>
+        <v>5.0599999999999999E-2</v>
       </c>
       <c r="S7" s="2">
-        <v>7.4649345331067485E-2</v>
+        <v>4.9799999999999997E-2</v>
       </c>
       <c r="T7" s="2">
-        <v>-0.12497102831907179</v>
+        <v>7.46E-2</v>
       </c>
       <c r="U7" s="2">
-        <v>-2.5217556612129769E-2</v>
+        <v>-0.125</v>
       </c>
       <c r="V7" s="2">
-        <v>0.10285331526718069</v>
+        <v>-2.52E-2</v>
       </c>
       <c r="W7" s="2">
-        <v>6.5038215096127949E-2</v>
+        <v>0.10290000000000001</v>
       </c>
       <c r="X7" s="2">
-        <v>1.2437482995890649E-2</v>
+        <v>6.5000000000000002E-2</v>
       </c>
       <c r="Y7" s="2">
-        <v>2.6700904863296241E-2</v>
+        <v>1.24E-2</v>
       </c>
       <c r="Z7" s="2">
-        <v>6.3062276236460102E-2</v>
+        <v>4.2299999999999997E-2</v>
       </c>
       <c r="AA7" s="2">
-        <v>-0.11689077106871799</v>
+        <v>6.3100000000000003E-2</v>
       </c>
       <c r="AB7" s="2">
-        <v>-2.5394156876443419E-2</v>
+        <v>-0.1169</v>
       </c>
       <c r="AC7" s="2">
-        <v>8.6757289789715752E-2</v>
+        <v>-2.5399999999999999E-2</v>
       </c>
       <c r="AD7" s="2">
-        <v>6.8712084440473165E-2</v>
+        <v>8.6800000000000002E-2</v>
       </c>
       <c r="AE7" s="2">
-        <v>1.4079379818825901E-2</v>
+        <v>6.8699999999999997E-2</v>
       </c>
       <c r="AF7" s="2">
-        <v>2.5157966737415108E-2</v>
+        <v>1.41E-2</v>
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
         <v>37</v>
       </c>
-      <c r="B8" t="s">
-        <v>38</v>
-      </c>
       <c r="C8" s="2">
-        <v>3.1978048780487711E-3</v>
+        <v>7.4000000000000003E-3</v>
       </c>
       <c r="D8" s="2">
-        <v>4.2031022549887657E-2</v>
+        <v>4.7800000000000002E-2</v>
       </c>
       <c r="E8" s="2">
-        <v>0.20212536985689011</v>
+        <v>0.2596</v>
       </c>
       <c r="F8" s="2">
-        <v>0.31065682515718279</v>
+        <v>0.2596</v>
       </c>
       <c r="G8" s="2">
-        <v>0.14079558605274919</v>
+        <v>0.1057</v>
       </c>
       <c r="H8" s="2">
-        <v>0.1236299658945996</v>
+        <v>0.13189999999999999</v>
       </c>
       <c r="I8" s="2">
-        <v>0.1177073111196925</v>
+        <v>0.1172</v>
       </c>
       <c r="J8" s="2">
-        <v>0.1041065210269836</v>
+        <v>0.1052</v>
       </c>
       <c r="K8" s="2">
-        <v>2.0699999999999941E-2</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="L8" s="2">
-        <v>5.0135314052000217E-2</v>
+        <v>6.2899999999999998E-2</v>
       </c>
       <c r="M8" s="2">
-        <v>0.2176712859544141</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="N8" s="2">
-        <v>0.32379111025699148</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="O8" s="2">
-        <v>0.11832710302928851</v>
+        <v>0.114</v>
       </c>
       <c r="P8" s="2">
-        <v>0.13733255744070519</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="Q8" s="2">
-        <v>0.12614947672235141</v>
+        <v>0.12770000000000001</v>
       </c>
       <c r="R8" s="2">
-        <v>9.1364002709943826E-2</v>
+        <v>9.3299999999999994E-2</v>
       </c>
       <c r="S8" s="2">
-        <v>0.1753993264425078</v>
+        <v>0.2596</v>
       </c>
       <c r="T8" s="2">
-        <v>-8.6883515521638199E-2</v>
+        <v>0.1754</v>
       </c>
       <c r="U8" s="2">
-        <v>0.26766545352246007</v>
+        <v>-8.6900000000000005E-2</v>
       </c>
       <c r="V8" s="2">
-        <v>8.4249303506370277E-2</v>
+        <v>0.26769999999999999</v>
       </c>
       <c r="W8" s="2">
-        <v>0.19638981733600039</v>
+        <v>8.4199999999999997E-2</v>
       </c>
       <c r="X8" s="2">
-        <v>-4.9599140354200646E-3</v>
+        <v>0.19639999999999999</v>
       </c>
       <c r="Y8" s="2">
-        <v>0.1307643627434181</v>
+        <v>-5.0000000000000001E-3</v>
       </c>
       <c r="Z8" s="2">
-        <v>0.21016918258785361</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="AA8" s="2">
-        <v>-0.1174573603921328</v>
+        <v>0.2102</v>
       </c>
       <c r="AB8" s="2">
-        <v>0.21310109733026381</v>
+        <v>-0.11749999999999999</v>
       </c>
       <c r="AC8" s="2">
-        <v>0.13322710348184111</v>
+        <v>0.21310000000000001</v>
       </c>
       <c r="AD8" s="2">
-        <v>0.21910476774026419</v>
+        <v>0.13320000000000001</v>
       </c>
       <c r="AE8" s="2">
-        <v>6.3113667818059938E-4</v>
+        <v>0.21909999999999999</v>
       </c>
       <c r="AF8" s="2">
-        <v>0.14987094927610209</v>
+        <v>5.9999999999999995E-4</v>
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" s="2">
-        <v>3.740607843137234E-3</v>
+        <v>4.4999999999999997E-3</v>
       </c>
       <c r="D9" s="2">
-        <v>4.2728367060641308E-2</v>
+        <v>4.7699999999999999E-2</v>
       </c>
       <c r="E9" s="2">
-        <v>0.2052482730798828</v>
+        <v>0.26279999999999998</v>
       </c>
       <c r="F9" s="2">
-        <v>0.31523973558142071</v>
+        <v>0.26279999999999998</v>
       </c>
       <c r="G9" s="2">
-        <v>0.14567254862590781</v>
+        <v>0.10299999999999999</v>
       </c>
       <c r="H9" s="2">
-        <v>0.1312942442029508</v>
+        <v>0.1384</v>
       </c>
       <c r="I9" s="2">
-        <v>0.1212642705491673</v>
+        <v>0.121</v>
       </c>
       <c r="J9" s="2">
-        <v>8.7964866834824518E-2</v>
+        <v>8.9599999999999999E-2</v>
       </c>
       <c r="K9" s="2">
-        <v>2.0699999999999941E-2</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="L9" s="2">
-        <v>5.0135314052000217E-2</v>
+        <v>6.2899999999999998E-2</v>
       </c>
       <c r="M9" s="2">
-        <v>0.2176712859544141</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="N9" s="2">
-        <v>0.32379111025699148</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="O9" s="2">
-        <v>0.11832710302928851</v>
+        <v>0.114</v>
       </c>
       <c r="P9" s="2">
-        <v>0.13733255744070519</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="Q9" s="2">
-        <v>0.12614947672235141</v>
+        <v>0.12770000000000001</v>
       </c>
       <c r="R9" s="2">
-        <v>9.7906926252477877E-2</v>
+        <v>0.1003</v>
       </c>
       <c r="S9" s="2">
-        <v>0.19210350219382619</v>
+        <v>0.26279999999999998</v>
       </c>
       <c r="T9" s="2">
-        <v>-0.1086485740791715</v>
+        <v>0.19209999999999999</v>
       </c>
       <c r="U9" s="2">
-        <v>0.31928245119478338</v>
+        <v>-0.1086</v>
       </c>
       <c r="V9" s="2">
-        <v>7.9992473769204819E-2</v>
+        <v>0.31929999999999997</v>
       </c>
       <c r="W9" s="2">
-        <v>0.2154545270790329</v>
+        <v>0.08</v>
       </c>
       <c r="X9" s="2">
-        <v>8.5866506209266724E-3</v>
+        <v>0.2155</v>
       </c>
       <c r="Y9" s="2">
-        <v>0.1168197181119066</v>
+        <v>8.6E-3</v>
       </c>
       <c r="Z9" s="2">
-        <v>0.21016918258785361</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="AA9" s="2">
-        <v>-0.1174573603921328</v>
+        <v>0.2102</v>
       </c>
       <c r="AB9" s="2">
-        <v>0.21310109733026381</v>
+        <v>-0.11749999999999999</v>
       </c>
       <c r="AC9" s="2">
-        <v>0.13322710348184111</v>
+        <v>0.21310000000000001</v>
       </c>
       <c r="AD9" s="2">
-        <v>0.21910476774026419</v>
+        <v>0.13320000000000001</v>
       </c>
       <c r="AE9" s="2">
-        <v>6.3113667818059938E-4</v>
+        <v>0.21909999999999999</v>
       </c>
       <c r="AF9" s="2">
-        <v>0.14987094927610209</v>
+        <v>5.9999999999999995E-4</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="B10" t="s">
-        <v>41</v>
-      </c>
       <c r="C10" s="2">
-        <v>3.0384777777777709E-2</v>
+        <v>-3.56E-2</v>
       </c>
       <c r="D10" s="2">
-        <v>0.10235523092467889</v>
+        <v>-1.0800000000000001E-2</v>
       </c>
       <c r="E10" s="2">
-        <v>0.1454098482651616</v>
+        <v>0.1331</v>
       </c>
       <c r="F10" s="2">
-        <v>0.24076789724687139</v>
+        <v>0.1331</v>
       </c>
       <c r="G10" s="2">
-        <v>0.1173705348296501</v>
+        <v>9.3799999999999994E-2</v>
       </c>
       <c r="H10" s="2">
-        <v>0.1104630532826678</v>
+        <v>9.9599999999999994E-2</v>
       </c>
       <c r="I10" s="2">
-        <v>7.3067843353594952E-2</v>
+        <v>7.5600000000000001E-2</v>
       </c>
       <c r="J10" s="2">
-        <v>0.1136995890506243</v>
+        <v>0.1118</v>
       </c>
       <c r="K10" s="2">
-        <v>3.5099999999999909E-2</v>
+        <v>-3.3399999999999999E-2</v>
       </c>
       <c r="L10" s="2">
-        <v>0.1164200955049999</v>
+        <v>7.7000000000000002E-3</v>
       </c>
       <c r="M10" s="2">
-        <v>0.14812411099481609</v>
+        <v>0.157</v>
       </c>
       <c r="N10" s="2">
-        <v>0.244686008261465</v>
+        <v>0.157</v>
       </c>
       <c r="O10" s="2">
-        <v>0.1029325233358485</v>
+        <v>7.9600000000000004E-2</v>
       </c>
       <c r="P10" s="2">
-        <v>0.1036181136168943</v>
+        <v>9.6600000000000005E-2</v>
       </c>
       <c r="Q10" s="2">
-        <v>7.0613369398904613E-2</v>
+        <v>7.7200000000000005E-2</v>
       </c>
       <c r="R10" s="2">
-        <v>0.1069262124947994</v>
+        <v>0.106</v>
       </c>
       <c r="S10" s="2">
-        <v>8.8744440171499184E-2</v>
+        <v>0.1331</v>
       </c>
       <c r="T10" s="2">
-        <v>6.0759705977495797E-2</v>
+        <v>8.8700000000000001E-2</v>
       </c>
       <c r="U10" s="2">
-        <v>0.30956324056409512</v>
+        <v>6.08E-2</v>
       </c>
       <c r="V10" s="2">
-        <v>-6.2025403848959597E-2</v>
+        <v>0.30959999999999999</v>
       </c>
       <c r="W10" s="2">
-        <v>0.2082705208707534</v>
+        <v>-6.2E-2</v>
       </c>
       <c r="X10" s="2">
-        <v>-0.1009024960682712</v>
+        <v>0.20830000000000001</v>
       </c>
       <c r="Y10" s="2">
-        <v>5.8599492359729721E-2</v>
+        <v>-0.1009</v>
       </c>
       <c r="Z10" s="2">
-        <v>8.050188529371205E-2</v>
+        <v>0.157</v>
       </c>
       <c r="AA10" s="2">
-        <v>6.431543794565231E-3</v>
+        <v>8.0500000000000002E-2</v>
       </c>
       <c r="AB10" s="2">
-        <v>0.36103956698877088</v>
+        <v>6.4000000000000003E-3</v>
       </c>
       <c r="AC10" s="2">
-        <v>-7.3860041217950645E-2</v>
+        <v>0.36099999999999999</v>
       </c>
       <c r="AD10" s="2">
-        <v>0.25812480061619558</v>
+        <v>-7.3899999999999993E-2</v>
       </c>
       <c r="AE10" s="2">
-        <v>-0.107731401591228</v>
+        <v>0.2581</v>
       </c>
       <c r="AF10" s="2">
-        <v>7.6128144206423665E-2</v>
+        <v>-0.1077</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" t="s">
         <v>42</v>
       </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
       <c r="C11" s="2">
-        <v>2.989568200836823E-2</v>
+        <v>-1.3100000000000001E-2</v>
       </c>
       <c r="D11" s="2">
-        <v>6.5185512421611413E-2</v>
+        <v>4.7699999999999999E-2</v>
       </c>
       <c r="E11" s="2">
-        <v>0.12930467673492621</v>
+        <v>0.1832</v>
       </c>
       <c r="F11" s="2">
-        <v>0.22349649546812439</v>
+        <v>0.1832</v>
       </c>
       <c r="G11" s="2">
-        <v>6.8468249791935332E-2</v>
+        <v>6.5000000000000002E-2</v>
       </c>
       <c r="H11" s="2">
-        <v>8.0055779828851481E-2</v>
+        <v>8.5800000000000001E-2</v>
       </c>
       <c r="I11" s="2">
-        <v>7.8751806289802273E-2</v>
+        <v>7.9500000000000001E-2</v>
       </c>
       <c r="J11" s="2">
-        <v>7.708003932822427E-2</v>
+        <v>7.8200000000000006E-2</v>
       </c>
       <c r="K11" s="2">
-        <v>2.3400000000000091E-2</v>
+        <v>-1.0999999999999999E-2</v>
       </c>
       <c r="L11" s="2">
-        <v>6.0901469600000091E-2</v>
+        <v>3.15E-2</v>
       </c>
       <c r="M11" s="2">
-        <v>0.1249954344629884</v>
+        <v>0.1605</v>
       </c>
       <c r="N11" s="2">
-        <v>0.21403848130129521</v>
+        <v>0.1605</v>
       </c>
       <c r="O11" s="2">
-        <v>5.8738780746780739E-2</v>
+        <v>5.2400000000000002E-2</v>
       </c>
       <c r="P11" s="2">
-        <v>7.2316384749006479E-2</v>
+        <v>7.46E-2</v>
       </c>
       <c r="Q11" s="2">
-        <v>7.1034847693849157E-2</v>
+        <v>7.0999999999999994E-2</v>
       </c>
       <c r="R11" s="2">
-        <v>7.0338801005845442E-2</v>
+        <v>7.0900000000000005E-2</v>
       </c>
       <c r="S11" s="2">
-        <v>0.17330481297705999</v>
+        <v>0.1832</v>
       </c>
       <c r="T11" s="2">
-        <v>-0.12996610793626931</v>
+        <v>0.17330000000000001</v>
       </c>
       <c r="U11" s="2">
-        <v>0.16260778923755589</v>
+        <v>-0.13</v>
       </c>
       <c r="V11" s="2">
-        <v>7.4865762310155848E-2</v>
+        <v>0.16259999999999999</v>
       </c>
       <c r="W11" s="2">
-        <v>0.12625265700684721</v>
+        <v>7.4899999999999994E-2</v>
       </c>
       <c r="X11" s="2">
-        <v>1.7279870544707251E-2</v>
+        <v>0.1263</v>
       </c>
       <c r="Y11" s="2">
-        <v>4.8745322067291319E-2</v>
+        <v>1.7299999999999999E-2</v>
       </c>
       <c r="Z11" s="2">
-        <v>0.1147928272931185</v>
+        <v>0.1605</v>
       </c>
       <c r="AA11" s="2">
-        <v>-9.9044415340767022E-2</v>
+        <v>0.1148</v>
       </c>
       <c r="AB11" s="2">
-        <v>0.112867795062521</v>
+        <v>-9.9000000000000005E-2</v>
       </c>
       <c r="AC11" s="2">
-        <v>0.1046288022437831</v>
+        <v>0.1129</v>
       </c>
       <c r="AD11" s="2">
-        <v>0.15197488384327329</v>
+        <v>0.1046</v>
       </c>
       <c r="AE11" s="2">
-        <v>-6.1622847520066406E-3</v>
+        <v>0.152</v>
       </c>
       <c r="AF11" s="2">
-        <v>6.9518674897322885E-2</v>
+        <v>-6.1999999999999998E-3</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
         <v>44</v>
       </c>
-      <c r="B12" t="s">
-        <v>45</v>
-      </c>
       <c r="C12" s="2">
-        <v>3.9075925373134313E-2</v>
+        <v>-1.7999999999999999E-2</v>
       </c>
       <c r="D12" s="2">
-        <v>7.6256850122417452E-2</v>
+        <v>7.5999999999999998E-2</v>
       </c>
       <c r="E12" s="2">
-        <v>0.19717887837264159</v>
+        <v>0.28820000000000001</v>
       </c>
       <c r="F12" s="2">
-        <v>0.3111762389766719</v>
+        <v>0.28820000000000001</v>
       </c>
       <c r="G12" s="2">
-        <v>0.116393212670183</v>
+        <v>0.11600000000000001</v>
       </c>
       <c r="H12" s="2">
-        <v>0.12664419633460261</v>
+        <v>0.13489999999999999</v>
       </c>
       <c r="I12" s="2">
-        <v>0.11185636511971039</v>
+        <v>0.1144</v>
       </c>
       <c r="J12" s="2">
-        <v>0.1005850076943124</v>
+        <v>0.10249999999999999</v>
       </c>
       <c r="K12" s="2">
-        <v>2.7700000000000061E-2</v>
+        <v>-1.4999999999999999E-2</v>
       </c>
       <c r="L12" s="2">
-        <v>7.5210272967000114E-2</v>
+        <v>6.3899999999999998E-2</v>
       </c>
       <c r="M12" s="2">
-        <v>0.2121435460487644</v>
+        <v>0.28960000000000002</v>
       </c>
       <c r="N12" s="2">
-        <v>0.31226991804058862</v>
+        <v>0.28960000000000002</v>
       </c>
       <c r="O12" s="2">
-        <v>0.1219940823067605</v>
+        <v>0.1144</v>
       </c>
       <c r="P12" s="2">
-        <v>0.13839584338095109</v>
+        <v>0.1414</v>
       </c>
       <c r="Q12" s="2">
-        <v>0.11925959760320649</v>
+        <v>0.1222</v>
       </c>
       <c r="R12" s="2">
-        <v>8.8634159765734077E-2</v>
+        <v>9.0200000000000002E-2</v>
       </c>
       <c r="S12" s="2">
-        <v>0.24089152985559159</v>
+        <v>0.28820000000000001</v>
       </c>
       <c r="T12" s="2">
-        <v>-0.13059519460896579</v>
+        <v>0.2409</v>
       </c>
       <c r="U12" s="2">
-        <v>0.25237616768120769</v>
+        <v>-0.13059999999999999</v>
       </c>
       <c r="V12" s="2">
-        <v>8.1569070295306689E-2</v>
+        <v>0.25240000000000001</v>
       </c>
       <c r="W12" s="2">
-        <v>0.1715094882487038</v>
+        <v>8.1600000000000006E-2</v>
       </c>
       <c r="X12" s="2">
-        <v>9.1529806240275846E-3</v>
+        <v>0.17150000000000001</v>
       </c>
       <c r="Y12" s="2">
-        <v>6.7357250409031622E-2</v>
+        <v>9.1999999999999998E-3</v>
       </c>
       <c r="Z12" s="2">
-        <v>0.1713694717429799</v>
+        <v>0.28960000000000002</v>
       </c>
       <c r="AA12" s="2">
-        <v>-8.3909329309362457E-2</v>
+        <v>0.1714</v>
       </c>
       <c r="AB12" s="2">
-        <v>0.26398989980912058</v>
+        <v>-8.3900000000000002E-2</v>
       </c>
       <c r="AC12" s="2">
-        <v>0.1075575934363073</v>
+        <v>0.26400000000000001</v>
       </c>
       <c r="AD12" s="2">
-        <v>0.23879323438722061</v>
+        <v>0.1076</v>
       </c>
       <c r="AE12" s="2">
-        <v>-2.4421037083545372E-2</v>
+        <v>0.23880000000000001</v>
       </c>
       <c r="AF12" s="2">
-        <v>0.114740125329617</v>
+        <v>-2.4400000000000002E-2</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" t="s">
         <v>46</v>
       </c>
-      <c r="B13" t="s">
-        <v>47</v>
-      </c>
       <c r="C13" s="2">
-        <v>1.223013846153842E-2</v>
+        <v>-1.04E-2</v>
       </c>
       <c r="D13" s="2">
-        <v>4.5058015671006313E-2</v>
+        <v>8.0600000000000005E-2</v>
       </c>
       <c r="E13" s="2">
-        <v>0.17867267387123539</v>
+        <v>0.2737</v>
       </c>
       <c r="F13" s="2">
-        <v>0.32074412636583788</v>
+        <v>0.2737</v>
       </c>
       <c r="G13" s="2">
-        <v>0.105965404068634</v>
+        <v>0.10440000000000001</v>
       </c>
       <c r="H13" s="2">
-        <v>0.16070620401157701</v>
+        <v>0.16619999999999999</v>
       </c>
       <c r="I13" s="2">
-        <v>0.1486894244440391</v>
+        <v>0.1515</v>
       </c>
       <c r="J13" s="2">
-        <v>9.8022825425732929E-2</v>
+        <v>0.10050000000000001</v>
       </c>
       <c r="K13" s="2">
-        <v>2.380000000000004E-2</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="L13" s="2">
-        <v>4.5488865146000153E-2</v>
+        <v>9.0300000000000005E-2</v>
       </c>
       <c r="M13" s="2">
-        <v>0.25087333727098637</v>
+        <v>0.36380000000000001</v>
       </c>
       <c r="N13" s="2">
-        <v>0.36147945571148238</v>
+        <v>0.36380000000000001</v>
       </c>
       <c r="O13" s="2">
-        <v>0.143150413533355</v>
+        <v>0.13730000000000001</v>
       </c>
       <c r="P13" s="2">
-        <v>0.16334525807966241</v>
+        <v>0.1681</v>
       </c>
       <c r="Q13" s="2">
-        <v>0.15493160358925581</v>
+        <v>0.1552</v>
       </c>
       <c r="R13" s="2">
-        <v>7.2453487737995426E-2</v>
+        <v>7.5499999999999998E-2</v>
       </c>
       <c r="S13" s="2">
-        <v>0.25428923880210452</v>
+        <v>0.2737</v>
       </c>
       <c r="T13" s="2">
-        <v>-0.15689063861803829</v>
+        <v>0.25430000000000003</v>
       </c>
       <c r="U13" s="2">
-        <v>0.27161910953713958</v>
+        <v>-0.15690000000000001</v>
       </c>
       <c r="V13" s="2">
-        <v>0.2595160966611858</v>
+        <v>0.27160000000000001</v>
       </c>
       <c r="W13" s="2">
-        <v>0.27375498705892748</v>
+        <v>0.25950000000000001</v>
       </c>
       <c r="X13" s="2">
-        <v>5.3456934933305167E-2</v>
+        <v>0.27379999999999999</v>
       </c>
       <c r="Y13" s="2">
-        <v>0.17685463127882509</v>
+        <v>5.3499999999999999E-2</v>
       </c>
       <c r="Z13" s="2">
-        <v>0.22802772224653481</v>
+        <v>0.36380000000000001</v>
       </c>
       <c r="AA13" s="2">
-        <v>-0.12152410109853</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="AB13" s="2">
-        <v>0.2761454551589928</v>
+        <v>-0.1215</v>
       </c>
       <c r="AC13" s="2">
-        <v>0.15829193424188981</v>
+        <v>0.27610000000000001</v>
       </c>
       <c r="AD13" s="2">
-        <v>0.24838940926861031</v>
+        <v>0.1583</v>
       </c>
       <c r="AE13" s="2">
-        <v>4.2275010225730332E-2</v>
+        <v>0.24840000000000001</v>
       </c>
       <c r="AF13" s="2">
-        <v>0.1382785534698816</v>
+        <v>4.2299999999999997E-2</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" s="2">
-        <v>2.5335450381679388E-2</v>
+        <v>-2.1600000000000001E-2</v>
       </c>
       <c r="D14" s="2">
-        <v>0.1063512739578658</v>
+        <v>1.9300000000000001E-2</v>
       </c>
       <c r="E14" s="2">
-        <v>0.17133660256431571</v>
+        <v>0.19389999999999999</v>
       </c>
       <c r="F14" s="2">
-        <v>0.23079951631181991</v>
+        <v>0.19389999999999999</v>
       </c>
       <c r="G14" s="2">
-        <v>0.117308611607428</v>
+        <v>9.8100000000000007E-2</v>
       </c>
       <c r="H14" s="2">
-        <v>0.1134806718616035</v>
+        <v>0.1096</v>
       </c>
       <c r="I14" s="2">
-        <v>7.8561348473661585E-2</v>
+        <v>7.9200000000000007E-2</v>
       </c>
       <c r="J14" s="2">
-        <v>0.1182540309999849</v>
+        <v>0.1179</v>
       </c>
       <c r="K14" s="2">
-        <v>3.1500000000000077E-2</v>
+        <v>-3.27E-2</v>
       </c>
       <c r="L14" s="2">
-        <v>0.10537204841</v>
+        <v>3.7699999999999997E-2</v>
       </c>
       <c r="M14" s="2">
-        <v>0.1722477759505909</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="N14" s="2">
-        <v>0.27034955217191731</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="O14" s="2">
-        <v>9.59203442098151E-2</v>
+        <v>8.6499999999999994E-2</v>
       </c>
       <c r="P14" s="2">
-        <v>0.1099255546061737</v>
+        <v>0.11119999999999999</v>
       </c>
       <c r="Q14" s="2">
-        <v>8.1103140812044172E-2</v>
+        <v>8.6699999999999999E-2</v>
       </c>
       <c r="R14" s="2">
-        <v>7.9825150528620714E-2</v>
+        <v>8.0600000000000005E-2</v>
       </c>
       <c r="S14" s="2">
-        <v>8.2265292556218395E-2</v>
+        <v>0.19389999999999999</v>
       </c>
       <c r="T14" s="2">
-        <v>2.4852794580773718E-2</v>
+        <v>8.2299999999999998E-2</v>
       </c>
       <c r="U14" s="2">
-        <v>0.28277174917337572</v>
+        <v>2.4899999999999999E-2</v>
       </c>
       <c r="V14" s="2">
-        <v>-9.987112125977915E-3</v>
+        <v>0.2828</v>
       </c>
       <c r="W14" s="2">
-        <v>0.20463900163792559</v>
+        <v>-0.01</v>
       </c>
       <c r="X14" s="2">
-        <v>-0.1130749971911198</v>
+        <v>0.2046</v>
       </c>
       <c r="Y14" s="2">
-        <v>5.2208536801292123E-2</v>
+        <v>-0.11310000000000001</v>
       </c>
       <c r="Z14" s="2">
-        <v>0.12021853546487481</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="AA14" s="2">
-        <v>-5.861422986020437E-2</v>
+        <v>0.1202</v>
       </c>
       <c r="AB14" s="2">
-        <v>0.25087973789207202</v>
+        <v>-5.8599999999999999E-2</v>
       </c>
       <c r="AC14" s="2">
-        <v>5.5915166451887321E-2</v>
+        <v>0.25090000000000001</v>
       </c>
       <c r="AD14" s="2">
-        <v>0.22876839007651761</v>
+        <v>5.5899999999999998E-2</v>
       </c>
       <c r="AE14" s="2">
-        <v>-8.8861093780151279E-2</v>
+        <v>0.2288</v>
       </c>
       <c r="AF14" s="2">
-        <v>9.0951444205845222E-2</v>
+        <v>-8.8900000000000007E-2</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" t="s">
         <v>49</v>
       </c>
-      <c r="B15" t="s">
-        <v>50</v>
-      </c>
       <c r="C15" s="2">
-        <v>1.6398700000000099E-2</v>
+        <v>-1.52E-2</v>
       </c>
       <c r="D15" s="2">
-        <v>7.9656922276349684E-2</v>
+        <v>1.0500000000000001E-2</v>
       </c>
       <c r="E15" s="2">
-        <v>0.1336010675431154</v>
+        <v>0.14549999999999999</v>
       </c>
       <c r="F15" s="2">
-        <v>0.2409925841349716</v>
+        <v>0.14549999999999999</v>
       </c>
       <c r="G15" s="2">
-        <v>9.834024759005211E-2</v>
+        <v>9.2499999999999999E-2</v>
       </c>
       <c r="H15" s="2">
-        <v>0.1226017923580804</v>
+        <v>0.1135</v>
       </c>
       <c r="I15" s="2">
-        <v>8.3460787109655099E-2</v>
+        <v>8.6800000000000002E-2</v>
       </c>
       <c r="J15" s="2">
-        <v>0.1129377927156836</v>
+        <v>0.1123</v>
       </c>
       <c r="K15" s="2">
-        <v>3.8000000000000027E-2</v>
+        <v>-3.3000000000000002E-2</v>
       </c>
       <c r="L15" s="2">
-        <v>8.4469121720000206E-2</v>
+        <v>6.7999999999999996E-3</v>
       </c>
       <c r="M15" s="2">
-        <v>0.1711383073572523</v>
+        <v>0.17910000000000001</v>
       </c>
       <c r="N15" s="2">
-        <v>0.2338624616364253</v>
+        <v>0.17910000000000001</v>
       </c>
       <c r="O15" s="2">
-        <v>4.7780518120132953E-2</v>
+        <v>3.8699999999999998E-2</v>
       </c>
       <c r="P15" s="2">
-        <v>0.1105438392491034</v>
+        <v>9.8599999999999993E-2</v>
       </c>
       <c r="Q15" s="2">
-        <v>5.97156579248459E-2</v>
+        <v>6.8500000000000005E-2</v>
       </c>
       <c r="R15" s="2">
-        <v>6.2921904795194994E-2</v>
+        <v>6.2600000000000003E-2</v>
       </c>
       <c r="S15" s="2">
-        <v>0.13163604439679649</v>
+        <v>0.14549999999999999</v>
       </c>
       <c r="T15" s="2">
-        <v>6.004942311459649E-3</v>
+        <v>0.13159999999999999</v>
       </c>
       <c r="U15" s="2">
-        <v>0.25963045708737781</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="V15" s="2">
-        <v>4.2266551135459629E-2</v>
+        <v>0.2596</v>
       </c>
       <c r="W15" s="2">
-        <v>0.174356775690232</v>
+        <v>4.2299999999999997E-2</v>
       </c>
       <c r="X15" s="2">
-        <v>-9.1042596803016851E-2</v>
+        <v>0.1744</v>
       </c>
       <c r="Y15" s="2">
-        <v>4.5366908340986001E-2</v>
+        <v>-9.0999999999999998E-2</v>
       </c>
       <c r="Z15" s="2">
-        <v>4.7003170409684943E-2</v>
+        <v>0.17910000000000001</v>
       </c>
       <c r="AA15" s="2">
-        <v>-9.2181445783686145E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="AB15" s="2">
-        <v>0.2479183845762456</v>
+        <v>-9.2200000000000004E-2</v>
       </c>
       <c r="AC15" s="2">
-        <v>0.14422856360136599</v>
+        <v>0.24790000000000001</v>
       </c>
       <c r="AD15" s="2">
-        <v>0.19203163120775571</v>
+        <v>0.14419999999999999</v>
       </c>
       <c r="AE15" s="2">
-        <v>-0.18167452986828991</v>
+        <v>0.192</v>
       </c>
       <c r="AF15" s="2">
-        <v>6.3764570033030266E-2</v>
+        <v>-0.1817</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C16" s="2">
-        <v>2.7499555555555499E-2</v>
+        <v>-3.1899999999999998E-2</v>
       </c>
       <c r="D16" s="2">
-        <v>0.11704385197475051</v>
+        <v>1.3599999999999999E-2</v>
       </c>
       <c r="E16" s="2">
-        <v>0.1631171957763913</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="F16" s="2">
-        <v>0.25614750571447908</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="G16" s="2">
-        <v>0.1214864631565606</v>
+        <v>9.6799999999999997E-2</v>
       </c>
       <c r="H16" s="2">
-        <v>0.1236969050181493</v>
+        <v>0.1206</v>
       </c>
       <c r="I16" s="2">
-        <v>8.931535120616374E-2</v>
+        <v>9.5299999999999996E-2</v>
       </c>
       <c r="J16" s="2">
-        <v>9.7577993576077215E-2</v>
+        <v>9.7199999999999995E-2</v>
       </c>
       <c r="K16" s="2">
-        <v>3.1500000000000077E-2</v>
+        <v>-3.27E-2</v>
       </c>
       <c r="L16" s="2">
-        <v>0.10537204841</v>
+        <v>3.7699999999999997E-2</v>
       </c>
       <c r="M16" s="2">
-        <v>0.1722477759505909</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="N16" s="2">
-        <v>0.27034955217191731</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="O16" s="2">
-        <v>9.59203442098151E-2</v>
+        <v>8.6499999999999994E-2</v>
       </c>
       <c r="P16" s="2">
-        <v>0.1099255546061737</v>
+        <v>0.11119999999999999</v>
       </c>
       <c r="Q16" s="2">
-        <v>8.1103140812044172E-2</v>
+        <v>8.6699999999999999E-2</v>
       </c>
       <c r="R16" s="2">
-        <v>7.3864750916512012E-2</v>
+        <v>7.46E-2</v>
       </c>
       <c r="S16" s="2">
-        <v>0.1026385713853166</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="T16" s="2">
-        <v>1.4977591714025349E-2</v>
+        <v>0.1026</v>
       </c>
       <c r="U16" s="2">
-        <v>0.3011668696139127</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="V16" s="2">
-        <v>2.9379985875004119E-2</v>
+        <v>0.30120000000000002</v>
       </c>
       <c r="W16" s="2">
-        <v>0.2051281246826844</v>
+        <v>2.9399999999999999E-2</v>
       </c>
       <c r="X16" s="2">
-        <v>-0.10290435971538731</v>
+        <v>0.2051</v>
       </c>
       <c r="Y16" s="2">
-        <v>0.10552560664093449</v>
+        <v>-0.10290000000000001</v>
       </c>
       <c r="Z16" s="2">
-        <v>0.12021853546487481</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="AA16" s="2">
-        <v>-5.861422986020437E-2</v>
+        <v>0.1202</v>
       </c>
       <c r="AB16" s="2">
-        <v>0.25087973789207202</v>
+        <v>-5.8599999999999999E-2</v>
       </c>
       <c r="AC16" s="2">
-        <v>5.5915166451887321E-2</v>
+        <v>0.25090000000000001</v>
       </c>
       <c r="AD16" s="2">
-        <v>0.22876839007651761</v>
+        <v>5.5899999999999998E-2</v>
       </c>
       <c r="AE16" s="2">
-        <v>-8.8861093780151279E-2</v>
+        <v>0.2288</v>
       </c>
       <c r="AF16" s="2">
-        <v>9.0951444205845222E-2</v>
+        <v>-8.8900000000000007E-2</v>
       </c>
     </row>
     <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" t="s">
         <v>52</v>
       </c>
-      <c r="B17" t="s">
-        <v>53</v>
-      </c>
       <c r="C17" s="2">
-        <v>1.6214539682539719E-2</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="D17" s="2">
-        <v>3.9770098030999852E-2</v>
+        <v>2.7799999999999998E-2</v>
       </c>
       <c r="E17" s="2">
-        <v>0.16023984955446521</v>
+        <v>0.1925</v>
       </c>
       <c r="F17" s="2">
-        <v>0.26827498429953378</v>
+        <v>0.1925</v>
       </c>
       <c r="G17" s="2">
-        <v>7.930351983261863E-2</v>
+        <v>6.2300000000000001E-2</v>
       </c>
       <c r="H17" s="2">
-        <v>0.1033947624028264</v>
+        <v>0.1026</v>
       </c>
       <c r="I17" s="2">
-        <v>0.11610764500069989</v>
+        <v>0.11210000000000001</v>
       </c>
       <c r="J17" s="2">
-        <v>8.1904280790688677E-2</v>
+        <v>8.2299999999999998E-2</v>
       </c>
       <c r="K17" s="2">
-        <v>2.570000000000006E-2</v>
+        <v>2.8999999999999998E-3</v>
       </c>
       <c r="L17" s="2">
-        <v>5.2686536252000149E-2</v>
+        <v>5.4100000000000002E-2</v>
       </c>
       <c r="M17" s="2">
-        <v>0.21575939086896631</v>
+        <v>0.28149999999999997</v>
       </c>
       <c r="N17" s="2">
-        <v>0.3182131747782746</v>
+        <v>0.28149999999999997</v>
       </c>
       <c r="O17" s="2">
-        <v>0.1048173625855031</v>
+        <v>0.10150000000000001</v>
       </c>
       <c r="P17" s="2">
-        <v>0.12284592008563421</v>
+        <v>0.1201</v>
       </c>
       <c r="Q17" s="2">
-        <v>0.1130330929084704</v>
+        <v>0.1145</v>
       </c>
       <c r="R17" s="2">
-        <v>8.0149043736965853E-2</v>
+        <v>8.1799999999999998E-2</v>
       </c>
       <c r="S17" s="2">
-        <v>0.14144707145853319</v>
+        <v>0.1925</v>
       </c>
       <c r="T17" s="2">
-        <v>-0.119339609569489</v>
+        <v>0.1414</v>
       </c>
       <c r="U17" s="2">
-        <v>0.17776070452224821</v>
+        <v>-0.1193</v>
       </c>
       <c r="V17" s="2">
-        <v>0.15429357627026061</v>
+        <v>0.17780000000000001</v>
       </c>
       <c r="W17" s="2">
-        <v>0.19951799007801679</v>
+        <v>0.15429999999999999</v>
       </c>
       <c r="X17" s="2">
-        <v>1.175024958400717E-2</v>
+        <v>0.19950000000000001</v>
       </c>
       <c r="Y17" s="2">
-        <v>0.18948574427267539</v>
+        <v>1.18E-2</v>
       </c>
       <c r="Z17" s="2">
-        <v>0.19088023426714379</v>
+        <v>0.28149999999999997</v>
       </c>
       <c r="AA17" s="2">
-        <v>-0.1242951408520198</v>
+        <v>0.19089999999999999</v>
       </c>
       <c r="AB17" s="2">
-        <v>0.17523622407634301</v>
+        <v>-0.12429999999999999</v>
       </c>
       <c r="AC17" s="2">
-        <v>0.1225417737020502</v>
+        <v>0.17519999999999999</v>
       </c>
       <c r="AD17" s="2">
-        <v>0.2019868939492451</v>
+        <v>0.1225</v>
       </c>
       <c r="AE17" s="2">
-        <v>-1.2569244036318761E-2</v>
+        <v>0.20200000000000001</v>
       </c>
       <c r="AF17" s="2">
-        <v>0.15828988716335449</v>
+        <v>-1.26E-2</v>
       </c>
     </row>
     <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" t="s">
         <v>54</v>
       </c>
-      <c r="B18" t="s">
-        <v>55</v>
-      </c>
       <c r="C18" s="2">
-        <v>1.397479999999995E-2</v>
+        <v>-7.1999999999999998E-3</v>
       </c>
       <c r="D18" s="2">
-        <v>8.3897361890910904E-2</v>
+        <v>-3.7999999999999999E-2</v>
       </c>
       <c r="E18" s="2">
-        <v>0.16828351529378521</v>
+        <v>0.12379999999999999</v>
       </c>
       <c r="F18" s="2">
-        <v>0.25951114653878887</v>
+        <v>0.12379999999999999</v>
       </c>
       <c r="G18" s="2">
-        <v>6.3394815593488696E-2</v>
+        <v>4.4699999999999997E-2</v>
       </c>
       <c r="H18" s="2">
-        <v>7.0749707688607888E-2</v>
+        <v>5.4600000000000003E-2</v>
       </c>
       <c r="I18" s="2">
-        <v>5.9662910661953061E-2</v>
+        <v>5.9400000000000001E-2</v>
       </c>
       <c r="J18" s="2">
-        <v>6.6578098457949375E-2</v>
+        <v>6.1499999999999999E-2</v>
       </c>
       <c r="K18" s="2">
-        <v>1.2000000000000011E-2</v>
+        <v>4.1000000000000003E-3</v>
       </c>
       <c r="L18" s="2">
-        <v>5.9557928000000038E-2</v>
+        <v>-2.1100000000000001E-2</v>
       </c>
       <c r="M18" s="2">
-        <v>0.16265099272484229</v>
+        <v>0.1381</v>
       </c>
       <c r="N18" s="2">
-        <v>0.25256683404955238</v>
+        <v>0.1381</v>
       </c>
       <c r="O18" s="2">
-        <v>8.3097067629413157E-2</v>
+        <v>6.6799999999999998E-2</v>
       </c>
       <c r="P18" s="2">
-        <v>8.948890540373089E-2</v>
+        <v>7.2300000000000003E-2</v>
       </c>
       <c r="Q18" s="2">
-        <v>6.7634228159824561E-2</v>
+        <v>6.9199999999999998E-2</v>
       </c>
       <c r="R18" s="2">
-        <v>7.4226944774093528E-2</v>
+        <v>7.0599999999999996E-2</v>
       </c>
       <c r="S18" s="2">
-        <v>0.1603299067404467</v>
+        <v>0.12379999999999999</v>
       </c>
       <c r="T18" s="2">
-        <v>-0.12561674946454729</v>
+        <v>0.1603</v>
       </c>
       <c r="U18" s="2">
-        <v>4.8196984917406649E-2</v>
+        <v>-0.12559999999999999</v>
       </c>
       <c r="V18" s="2">
-        <v>9.1570236649640702E-2</v>
+        <v>4.82E-2</v>
       </c>
       <c r="W18" s="2">
-        <v>0.14015252299746009</v>
+        <v>9.1600000000000001E-2</v>
       </c>
       <c r="X18" s="2">
-        <v>-7.2063760598472859E-2</v>
+        <v>0.14019999999999999</v>
       </c>
       <c r="Y18" s="2">
-        <v>0.27680869263481078</v>
+        <v>-7.2099999999999997E-2</v>
       </c>
       <c r="Z18" s="2">
-        <v>0.1566567055638326</v>
+        <v>0.1381</v>
       </c>
       <c r="AA18" s="2">
-        <v>-7.7705292109581325E-2</v>
+        <v>0.15670000000000001</v>
       </c>
       <c r="AB18" s="2">
-        <v>0.10817931502983601</v>
+        <v>-7.7700000000000005E-2</v>
       </c>
       <c r="AC18" s="2">
-        <v>5.377222737175158E-2</v>
+        <v>0.1082</v>
       </c>
       <c r="AD18" s="2">
-        <v>0.1645435923658487</v>
+        <v>5.3800000000000001E-2</v>
       </c>
       <c r="AE18" s="2">
-        <v>-5.5537819245731417E-2</v>
+        <v>0.16450000000000001</v>
       </c>
       <c r="AF18" s="2">
-        <v>0.25034361477208772</v>
+        <v>-5.5500000000000001E-2</v>
       </c>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C19" s="2">
-        <v>1.7886466666666712E-2</v>
+        <v>-2.3300000000000001E-2</v>
       </c>
       <c r="D19" s="2">
-        <v>8.8768277783860317E-2</v>
+        <v>2.69E-2</v>
       </c>
       <c r="E19" s="2">
-        <v>0.1399681011970324</v>
+        <v>0.1706</v>
       </c>
       <c r="F19" s="2">
-        <v>0.21102943559301621</v>
+        <v>0.1706</v>
       </c>
       <c r="G19" s="2">
-        <v>0.13324976351563089</v>
+        <v>0.11700000000000001</v>
       </c>
       <c r="H19" s="2">
-        <v>0.1098552414969942</v>
+        <v>0.112</v>
       </c>
       <c r="I19" s="2">
-        <v>8.3681481721308071E-2</v>
+        <v>8.8200000000000001E-2</v>
       </c>
       <c r="J19" s="2">
-        <v>8.5298665128509921E-2</v>
+        <v>8.5599999999999996E-2</v>
       </c>
       <c r="K19" s="2">
-        <v>3.1500000000000077E-2</v>
+        <v>-3.27E-2</v>
       </c>
       <c r="L19" s="2">
-        <v>0.10537204841</v>
+        <v>3.7699999999999997E-2</v>
       </c>
       <c r="M19" s="2">
-        <v>0.1722477759505909</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="N19" s="2">
-        <v>0.27034955217191731</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="O19" s="2">
-        <v>9.59203442098151E-2</v>
+        <v>8.6499999999999994E-2</v>
       </c>
       <c r="P19" s="2">
-        <v>0.1099255546061737</v>
+        <v>0.11119999999999999</v>
       </c>
       <c r="Q19" s="2">
-        <v>8.1103140812044172E-2</v>
+        <v>8.6699999999999999E-2</v>
       </c>
       <c r="R19" s="2">
-        <v>8.0315318049467566E-2</v>
+        <v>8.1299999999999997E-2</v>
       </c>
       <c r="S19" s="2">
-        <v>0.10821411542389291</v>
+        <v>0.1706</v>
       </c>
       <c r="T19" s="2">
-        <v>7.4346142515499869E-2</v>
+        <v>0.1082</v>
       </c>
       <c r="U19" s="2">
-        <v>0.22162757928016791</v>
+        <v>7.4300000000000005E-2</v>
       </c>
       <c r="V19" s="2">
-        <v>-1.452798809084666E-3</v>
+        <v>0.22159999999999999</v>
       </c>
       <c r="W19" s="2">
-        <v>0.1855372953368859</v>
+        <v>-1.5E-3</v>
       </c>
       <c r="X19" s="2">
-        <v>-9.8920016607088379E-2</v>
+        <v>0.1855</v>
       </c>
       <c r="Y19" s="2">
-        <v>0.1052521249019638</v>
+        <v>-9.8900000000000002E-2</v>
       </c>
       <c r="Z19" s="2">
-        <v>0.12021853546487481</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="AA19" s="2">
-        <v>-5.861422986020437E-2</v>
+        <v>0.1202</v>
       </c>
       <c r="AB19" s="2">
-        <v>0.25087973789207202</v>
+        <v>-5.8599999999999999E-2</v>
       </c>
       <c r="AC19" s="2">
-        <v>5.5915166451887321E-2</v>
+        <v>0.25090000000000001</v>
       </c>
       <c r="AD19" s="2">
-        <v>0.22876839007651761</v>
+        <v>5.5899999999999998E-2</v>
       </c>
       <c r="AE19" s="2">
-        <v>-8.8861093780151279E-2</v>
+        <v>0.2288</v>
       </c>
       <c r="AF19" s="2">
-        <v>9.0951444205845222E-2</v>
+        <v>-8.8900000000000007E-2</v>
       </c>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C20" s="2">
-        <v>3.2473600000000102E-2</v>
+        <v>-3.9100000000000003E-2</v>
       </c>
       <c r="D20" s="2">
-        <v>0.10321088885485021</v>
+        <v>6.4000000000000003E-3</v>
       </c>
       <c r="E20" s="2">
-        <v>0.20920028093181339</v>
+        <v>0.21690000000000001</v>
       </c>
       <c r="F20" s="2">
-        <v>0.31176511676575958</v>
+        <v>0.21690000000000001</v>
       </c>
       <c r="G20" s="2">
-        <v>0.1216048730670725</v>
+        <v>9.8299999999999998E-2</v>
       </c>
       <c r="H20" s="2">
-        <v>0.1141511986577102</v>
+        <v>0.1125</v>
       </c>
       <c r="I20" s="2">
-        <v>8.9484920299482962E-2</v>
+        <v>8.9599999999999999E-2</v>
       </c>
       <c r="J20" s="2">
-        <v>8.4689087336725422E-2</v>
+        <v>8.3599999999999994E-2</v>
       </c>
       <c r="K20" s="2">
-        <v>3.1500000000000077E-2</v>
+        <v>-3.27E-2</v>
       </c>
       <c r="L20" s="2">
-        <v>0.10537204841</v>
+        <v>3.7699999999999997E-2</v>
       </c>
       <c r="M20" s="2">
-        <v>0.1722477759505909</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="N20" s="2">
-        <v>0.27034955217191731</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="O20" s="2">
-        <v>9.59203442098151E-2</v>
+        <v>8.6499999999999994E-2</v>
       </c>
       <c r="P20" s="2">
-        <v>0.1099255546061737</v>
+        <v>0.11119999999999999</v>
       </c>
       <c r="Q20" s="2">
-        <v>8.1103140812044172E-2</v>
+        <v>8.6699999999999999E-2</v>
       </c>
       <c r="R20" s="2">
-        <v>7.3110292664734233E-2</v>
+        <v>7.46E-2</v>
       </c>
       <c r="S20" s="2">
-        <v>0.16128355856189081</v>
+        <v>0.21690000000000001</v>
       </c>
       <c r="T20" s="2">
-        <v>-6.265463117122505E-2</v>
+        <v>0.1613</v>
       </c>
       <c r="U20" s="2">
-        <v>0.2345884019388873</v>
+        <v>-6.2700000000000006E-2</v>
       </c>
       <c r="V20" s="2">
-        <v>4.1925939270043289E-2</v>
+        <v>0.2346</v>
       </c>
       <c r="W20" s="2">
-        <v>0.1841829826693191</v>
+        <v>4.19E-2</v>
       </c>
       <c r="X20" s="2">
-        <v>-6.4730847858231022E-2</v>
+        <v>0.1842</v>
       </c>
       <c r="Y20" s="2">
-        <v>9.2532317852311641E-2</v>
+        <v>-6.4699999999999994E-2</v>
       </c>
       <c r="Z20" s="2">
-        <v>0.12021853546487481</v>
+        <v>0.21640000000000001</v>
       </c>
       <c r="AA20" s="2">
-        <v>-5.861422986020437E-2</v>
+        <v>0.1202</v>
       </c>
       <c r="AB20" s="2">
-        <v>0.25087973789207202</v>
+        <v>-5.8599999999999999E-2</v>
       </c>
       <c r="AC20" s="2">
-        <v>5.5915166451887321E-2</v>
+        <v>0.25090000000000001</v>
       </c>
       <c r="AD20" s="2">
-        <v>0.22876839007651761</v>
+        <v>5.5899999999999998E-2</v>
       </c>
       <c r="AE20" s="2">
-        <v>-8.8861093780151279E-2</v>
+        <v>0.2288</v>
       </c>
       <c r="AF20" s="2">
-        <v>9.0951444205845222E-2</v>
+        <v>-8.8900000000000007E-2</v>
       </c>
     </row>
     <row r="21" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C21" s="2">
-        <v>2.0495699999999891E-2</v>
+        <v>-6.7999999999999996E-3</v>
       </c>
       <c r="D21" s="2">
-        <v>5.1662501027481163E-2</v>
+        <v>-5.9999999999999995E-4</v>
       </c>
       <c r="E21" s="2">
-        <v>4.8447341832999813E-2</v>
+        <v>4.7800000000000002E-2</v>
       </c>
       <c r="F21" s="2">
-        <v>0.14157302505347499</v>
+        <v>4.7800000000000002E-2</v>
       </c>
       <c r="G21" s="2">
-        <v>3.6224476966539849E-3</v>
+        <v>-1.1999999999999999E-3</v>
       </c>
       <c r="H21" s="2">
-        <v>1.042862737329564E-2</v>
+        <v>1.3599999999999999E-2</v>
       </c>
       <c r="I21" s="2">
-        <v>2.6186751368436401E-2</v>
+        <v>2.47E-2</v>
       </c>
       <c r="J21" s="2">
-        <v>2.751394192597378E-2</v>
+        <v>2.7E-2</v>
       </c>
       <c r="K21" s="2">
-        <v>1.9099999999999891E-2</v>
+        <v>-6.8999999999999999E-3</v>
       </c>
       <c r="L21" s="2">
-        <v>4.659107854400002E-2</v>
+        <v>-5.0000000000000001E-4</v>
       </c>
       <c r="M21" s="2">
-        <v>4.2794816038896011E-2</v>
+        <v>4.2299999999999997E-2</v>
       </c>
       <c r="N21" s="2">
-        <v>0.124976108740396</v>
+        <v>4.2299999999999997E-2</v>
       </c>
       <c r="O21" s="2">
-        <v>-2.2046397650784528E-3</v>
+        <v>-7.1999999999999998E-3</v>
       </c>
       <c r="P21" s="2">
-        <v>5.5507327550163854E-3</v>
+        <v>7.1999999999999998E-3</v>
       </c>
       <c r="Q21" s="2">
-        <v>2.2170375268985461E-2</v>
+        <v>1.9400000000000001E-2</v>
       </c>
       <c r="R21" s="2">
-        <v>2.9486948262095639E-2</v>
+        <v>2.8899999999999999E-2</v>
       </c>
       <c r="S21" s="2">
-        <v>7.1266059690755723E-2</v>
+        <v>4.7800000000000002E-2</v>
       </c>
       <c r="T21" s="2">
-        <v>-0.1122760042000059</v>
+        <v>7.1300000000000002E-2</v>
       </c>
       <c r="U21" s="2">
-        <v>-2.948019697857374E-2</v>
+        <v>-0.1123</v>
       </c>
       <c r="V21" s="2">
-        <v>0.106471440358697</v>
+        <v>-2.9499999999999998E-2</v>
       </c>
       <c r="W21" s="2">
-        <v>5.9792896594321743E-2</v>
+        <v>0.1065</v>
       </c>
       <c r="X21" s="2">
-        <v>2.3394529554544349E-2</v>
+        <v>5.9799999999999999E-2</v>
       </c>
       <c r="Y21" s="2">
-        <v>4.5088281973713507E-2</v>
+        <v>2.3400000000000001E-2</v>
       </c>
       <c r="Z21" s="2">
-        <v>6.3062276236460102E-2</v>
+        <v>4.2299999999999997E-2</v>
       </c>
       <c r="AA21" s="2">
-        <v>-0.11689077106871799</v>
+        <v>6.3100000000000003E-2</v>
       </c>
       <c r="AB21" s="2">
-        <v>-2.5394156876443419E-2</v>
+        <v>-0.1169</v>
       </c>
       <c r="AC21" s="2">
-        <v>8.6757289789715752E-2</v>
+        <v>-2.5399999999999999E-2</v>
       </c>
       <c r="AD21" s="2">
-        <v>6.8712084440473165E-2</v>
+        <v>8.6800000000000002E-2</v>
       </c>
       <c r="AE21" s="2">
-        <v>1.4079379818825901E-2</v>
+        <v>6.8699999999999997E-2</v>
       </c>
       <c r="AF21" s="2">
-        <v>2.5157966737415108E-2</v>
+        <v>1.41E-2</v>
       </c>
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" t="s">
         <v>59</v>
       </c>
-      <c r="B22" t="s">
-        <v>60</v>
-      </c>
       <c r="C22" s="2">
-        <v>1.9037399999999979E-2</v>
+        <v>-7.4000000000000003E-3</v>
       </c>
       <c r="D22" s="2">
-        <v>6.1643979382963732E-2</v>
+        <v>3.4299999999999997E-2</v>
       </c>
       <c r="E22" s="2">
-        <v>0.14551616196982239</v>
+        <v>0.18479999999999999</v>
       </c>
       <c r="F22" s="2">
-        <v>0.2469875099793741</v>
+        <v>0.18479999999999999</v>
       </c>
       <c r="G22" s="2">
-        <v>7.5962953156142321E-2</v>
+        <v>6.4799999999999996E-2</v>
       </c>
       <c r="H22" s="2">
-        <v>0.1141364343583384</v>
+        <v>0.1195</v>
       </c>
       <c r="I22" s="2">
-        <v>8.9343217834835453E-2</v>
+        <v>9.0399999999999994E-2</v>
       </c>
       <c r="J22" s="2">
-        <v>7.7727198535543662E-2</v>
+        <v>7.8899999999999998E-2</v>
       </c>
       <c r="K22" s="2">
-        <v>2.3300000000000098E-2</v>
+        <v>-1.2500000000000001E-2</v>
       </c>
       <c r="L22" s="2">
-        <v>6.5143371445999909E-2</v>
+        <v>2.9899999999999999E-2</v>
       </c>
       <c r="M22" s="2">
-        <v>0.1324220958741584</v>
+        <v>0.1663</v>
       </c>
       <c r="N22" s="2">
-        <v>0.2277637172169997</v>
+        <v>0.1663</v>
       </c>
       <c r="O22" s="2">
-        <v>6.4493775181033941E-2</v>
+        <v>5.7099999999999998E-2</v>
       </c>
       <c r="P22" s="2">
-        <v>7.798992249840131E-2</v>
+        <v>7.9399999999999998E-2</v>
       </c>
       <c r="Q22" s="2">
-        <v>7.3571064936981845E-2</v>
+        <v>7.4200000000000002E-2</v>
       </c>
       <c r="R22" s="2">
-        <v>7.4850483099118348E-2</v>
+        <v>7.5700000000000003E-2</v>
       </c>
       <c r="S22" s="2">
-        <v>0.14129585786912119</v>
+        <v>0.18479999999999999</v>
       </c>
       <c r="T22" s="2">
-        <v>-0.10715189023336751</v>
+        <v>0.14130000000000001</v>
       </c>
       <c r="U22" s="2">
-        <v>0.1390876955281328</v>
+        <v>-0.1072</v>
       </c>
       <c r="V22" s="2">
-        <v>0.27876690576895458</v>
+        <v>0.1391</v>
       </c>
       <c r="W22" s="2">
-        <v>0.12965554966895601</v>
+        <v>0.27879999999999999</v>
       </c>
       <c r="X22" s="2">
-        <v>-2.6555424912946379E-2</v>
+        <v>0.12970000000000001</v>
       </c>
       <c r="Y22" s="2">
-        <v>8.5428820062357858E-2</v>
+        <v>-2.6599999999999999E-2</v>
       </c>
       <c r="Z22" s="2">
-        <v>0.1240317190194777</v>
+        <v>0.1663</v>
       </c>
       <c r="AA22" s="2">
-        <v>-9.8973580499673863E-2</v>
+        <v>0.124</v>
       </c>
       <c r="AB22" s="2">
-        <v>0.1310961488382727</v>
+        <v>-9.9000000000000005E-2</v>
       </c>
       <c r="AC22" s="2">
-        <v>9.6828978745500338E-2</v>
+        <v>0.13109999999999999</v>
       </c>
       <c r="AD22" s="2">
-        <v>0.1578400001663933</v>
+        <v>9.6799999999999997E-2</v>
       </c>
       <c r="AE22" s="2">
-        <v>-1.6408690648921479E-2</v>
+        <v>0.1578</v>
       </c>
       <c r="AF22" s="2">
-        <v>8.3512134670415517E-2</v>
+        <v>-1.6400000000000001E-2</v>
       </c>
     </row>
     <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C23" s="2">
-        <v>1.1731999999999849E-3</v>
+        <v>6.7000000000000002E-3</v>
       </c>
       <c r="D23" s="2">
-        <v>3.9468291033270431E-2</v>
+        <v>4.8300000000000003E-2</v>
       </c>
       <c r="E23" s="2">
-        <v>0.20879827581818411</v>
+        <v>0.26719999999999999</v>
       </c>
       <c r="F23" s="2">
-        <v>0.31373890477876909</v>
+        <v>0.26719999999999999</v>
       </c>
       <c r="G23" s="2">
-        <v>0.14543236136054261</v>
+        <v>0.11070000000000001</v>
       </c>
       <c r="H23" s="2">
-        <v>0.12517652202644541</v>
+        <v>0.13200000000000001</v>
       </c>
       <c r="I23" s="2">
-        <v>0.1143443973527549</v>
+        <v>0.1129</v>
       </c>
       <c r="J23" s="2">
-        <v>0.111661502327461</v>
+        <v>0.1133</v>
       </c>
       <c r="K23" s="2">
-        <v>2.0699999999999941E-2</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="L23" s="2">
-        <v>5.0135314052000217E-2</v>
+        <v>6.2899999999999998E-2</v>
       </c>
       <c r="M23" s="2">
-        <v>0.2176712859544141</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="N23" s="2">
-        <v>0.32379111025699148</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="O23" s="2">
-        <v>0.11832710302928851</v>
+        <v>0.114</v>
       </c>
       <c r="P23" s="2">
-        <v>0.13733255744070519</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="Q23" s="2">
-        <v>0.12614947672235141</v>
+        <v>0.12770000000000001</v>
       </c>
       <c r="R23" s="2">
-        <v>0.13105623988740761</v>
+        <v>0.13350000000000001</v>
       </c>
       <c r="S23" s="2">
-        <v>0.17242431806507999</v>
+        <v>0.26719999999999999</v>
       </c>
       <c r="T23" s="2">
-        <v>-7.7608178432540642E-2</v>
+        <v>0.1724</v>
       </c>
       <c r="U23" s="2">
-        <v>0.2685087416826839</v>
+        <v>-7.7600000000000002E-2</v>
       </c>
       <c r="V23" s="2">
-        <v>6.9484493602757436E-2</v>
+        <v>0.26850000000000002</v>
       </c>
       <c r="W23" s="2">
-        <v>0.18579928386096009</v>
+        <v>6.9500000000000006E-2</v>
       </c>
       <c r="X23" s="2">
-        <v>-1.734092389593855E-2</v>
+        <v>0.18579999999999999</v>
       </c>
       <c r="Y23" s="2">
-        <v>0.14153247006992339</v>
+        <v>-1.7299999999999999E-2</v>
       </c>
       <c r="Z23" s="2">
-        <v>0.21016918258785361</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="AA23" s="2">
-        <v>-0.1174573603921328</v>
+        <v>0.2102</v>
       </c>
       <c r="AB23" s="2">
-        <v>0.21310109733026381</v>
+        <v>-0.11749999999999999</v>
       </c>
       <c r="AC23" s="2">
-        <v>0.13322710348184111</v>
+        <v>0.21310000000000001</v>
       </c>
       <c r="AD23" s="2">
-        <v>0.21910476774026419</v>
+        <v>0.13320000000000001</v>
       </c>
       <c r="AE23" s="2">
-        <v>6.3113667818059938E-4</v>
+        <v>0.21909999999999999</v>
       </c>
       <c r="AF23" s="2">
-        <v>0.14987094927610209</v>
+        <v>5.9999999999999995E-4</v>
       </c>
     </row>
     <row r="24" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C24" s="2">
-        <v>2.9416666666666666E-3</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="D24" s="2">
-        <v>8.8249999999999995E-3</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="E24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="F24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="G24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="H24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="I24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="J24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="K24" s="2">
-        <v>2.9416666666666666E-3</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="L24" s="2">
-        <v>8.8249999999999995E-3</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="M24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="N24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="O24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="P24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="Q24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="R24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="S24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="T24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="U24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="V24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="W24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="X24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="Y24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="Z24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="AA24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="AB24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="AC24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="AD24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="AE24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="AF24" s="2">
-        <v>3.5299999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
     </row>
     <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" t="s">
         <v>64</v>
       </c>
-      <c r="B25" t="s">
-        <v>65</v>
-      </c>
       <c r="C25" s="2">
-        <v>1.195352380952386E-2</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="D25" s="2">
-        <v>8.6750000000000004E-3</v>
+        <v>7.7999999999999996E-3</v>
       </c>
       <c r="E25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="F25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="G25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="H25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="I25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="J25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="K25" s="2">
-        <v>1.195352380952386E-2</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="L25" s="2">
-        <v>8.6750000000000004E-3</v>
+        <v>7.7999999999999996E-3</v>
       </c>
       <c r="M25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="N25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="O25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="P25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="Q25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="R25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="S25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="T25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="U25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="V25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="W25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="X25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="Y25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="Z25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="AA25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="AB25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="AC25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="AD25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="AE25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
       <c r="AF25" s="2">
-        <v>3.4700000000000002E-2</v>
+        <v>3.1699999999999999E-2</v>
       </c>
     </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C26" s="2">
-        <v>2.0699999999999941E-2</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="D26" s="2">
-        <v>5.0135314052000217E-2</v>
+        <v>6.2899999999999998E-2</v>
       </c>
       <c r="E26" s="2">
-        <v>0.2176712859544141</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="F26" s="2">
-        <v>0.32379111025699148</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="G26" s="2">
-        <v>0.11832710302928851</v>
+        <v>0.114</v>
       </c>
       <c r="H26" s="2">
-        <v>0.13733255744070519</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="I26" s="2">
-        <v>0.12614947672235141</v>
+        <v>0.12770000000000001</v>
       </c>
       <c r="J26" s="2">
-        <v>9.7906926252477877E-2</v>
+        <v>9.3299999999999994E-2</v>
       </c>
       <c r="K26" s="2">
-        <v>2.0699999999999941E-2</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="L26" s="2">
-        <v>5.0135314052000217E-2</v>
+        <v>6.2899999999999998E-2</v>
       </c>
       <c r="M26" s="2">
-        <v>0.2176712859544141</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="N26" s="2">
-        <v>0.32379111025699148</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="O26" s="2">
-        <v>0.11832710302928851</v>
+        <v>0.114</v>
       </c>
       <c r="P26" s="2">
-        <v>0.13733255744070519</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="Q26" s="2">
-        <v>0.12614947672235141</v>
+        <v>0.12770000000000001</v>
       </c>
       <c r="R26" s="2">
-        <v>9.7906926252477877E-2</v>
+        <v>9.3299999999999994E-2</v>
       </c>
       <c r="S26" s="2">
-        <v>0.21016918258785361</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="T26" s="2">
-        <v>-0.1174573603921328</v>
+        <v>0.2102</v>
       </c>
       <c r="U26" s="2">
-        <v>0.21310109733026381</v>
+        <v>-0.11749999999999999</v>
       </c>
       <c r="V26" s="2">
-        <v>0.13322710348184111</v>
+        <v>0.21310000000000001</v>
       </c>
       <c r="W26" s="2">
-        <v>0.21910476774026419</v>
+        <v>0.13320000000000001</v>
       </c>
       <c r="X26" s="2">
-        <v>6.3113667818059938E-4</v>
+        <v>0.21909999999999999</v>
       </c>
       <c r="Y26" s="2">
-        <v>0.14987094927610209</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="Z26" s="2">
-        <v>0.21016918258785361</v>
+        <v>0.29430000000000001</v>
       </c>
       <c r="AA26" s="2">
-        <v>-0.1174573603921328</v>
+        <v>0.2102</v>
       </c>
       <c r="AB26" s="2">
-        <v>0.21310109733026381</v>
+        <v>-0.11749999999999999</v>
       </c>
       <c r="AC26" s="2">
-        <v>0.13322710348184111</v>
+        <v>0.21310000000000001</v>
       </c>
       <c r="AD26" s="2">
-        <v>0.21910476774026419</v>
+        <v>0.13320000000000001</v>
       </c>
       <c r="AE26" s="2">
-        <v>6.3113667818059938E-4</v>
+        <v>0.21909999999999999</v>
       </c>
       <c r="AF26" s="2">
-        <v>0.14987094927610209</v>
+        <v>5.9999999999999995E-4</v>
       </c>
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" t="s">
         <v>62</v>
       </c>
-      <c r="B27" t="s">
-        <v>63</v>
-      </c>
-      <c r="C27">
-        <v>2.69E-2</v>
-      </c>
-      <c r="D27">
-        <v>7.749807401599984E-2</v>
-      </c>
-      <c r="E27">
-        <v>0.11097310282703532</v>
-      </c>
-      <c r="F27">
-        <v>0.18075718217010972</v>
-      </c>
-      <c r="G27">
-        <v>5.705508931930936E-2</v>
-      </c>
-      <c r="H27">
-        <v>5.3837254218028319E-2</v>
-      </c>
-      <c r="I27">
-        <v>5.557549702237341E-2</v>
-      </c>
-      <c r="J27">
-        <v>6.3386412215678645E-2</v>
-      </c>
-      <c r="K27">
-        <v>2.69E-2</v>
-      </c>
-      <c r="L27">
-        <v>7.749807401599984E-2</v>
-      </c>
-      <c r="M27">
-        <v>0.11097310282703532</v>
-      </c>
-      <c r="N27">
-        <v>0.18075718217010972</v>
-      </c>
-      <c r="O27">
-        <v>5.705508931930936E-2</v>
-      </c>
-      <c r="P27">
-        <v>5.3837254218028319E-2</v>
-      </c>
-      <c r="Q27">
-        <v>5.557549702237341E-2</v>
-      </c>
-      <c r="R27">
-        <v>6.3386412215678645E-2</v>
-      </c>
-      <c r="S27">
-        <v>5.4098630863060437E-2</v>
-      </c>
-      <c r="T27">
-        <v>-3.42026528470857E-2</v>
-      </c>
-      <c r="U27">
-        <v>0.1455653061407236</v>
-      </c>
-      <c r="V27">
-        <v>-8.3092281574879134E-3</v>
-      </c>
-      <c r="W27">
-        <v>0.115914764648821</v>
-      </c>
-      <c r="X27">
-        <v>2.0091365915979598E-2</v>
-      </c>
-      <c r="Y27">
-        <v>4.1013315214144752E-2</v>
-      </c>
-      <c r="Z27">
-        <v>5.4098630863060437E-2</v>
-      </c>
-      <c r="AA27">
-        <v>-3.4202652847085679E-2</v>
-      </c>
-      <c r="AB27">
-        <v>0.1455653061407236</v>
-      </c>
-      <c r="AC27">
-        <v>-8.3092281574879134E-3</v>
-      </c>
-      <c r="AD27">
-        <v>0.115914764648821</v>
-      </c>
-      <c r="AE27">
-        <v>2.0091365915979598E-2</v>
-      </c>
-      <c r="AF27">
-        <v>4.1013315214144752E-2</v>
+      <c r="C27" s="3">
+        <v>-1.11E-2</v>
+      </c>
+      <c r="D27" s="3">
+        <v>1.24E-2</v>
+      </c>
+      <c r="E27" s="3">
+        <v>0.12479999999999999</v>
+      </c>
+      <c r="F27" s="3">
+        <v>0.12479999999999999</v>
+      </c>
+      <c r="G27" s="3">
+        <v>4.6199999999999998E-2</v>
+      </c>
+      <c r="H27" s="3">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="I27" s="3">
+        <v>5.5599999999999997E-2</v>
+      </c>
+      <c r="J27" s="3">
+        <v>6.3200000000000006E-2</v>
+      </c>
+      <c r="K27" s="3">
+        <v>-1.11E-2</v>
+      </c>
+      <c r="L27" s="3">
+        <v>1.24E-2</v>
+      </c>
+      <c r="M27" s="3">
+        <v>0.12479999999999999</v>
+      </c>
+      <c r="N27" s="3">
+        <v>0.12479999999999999</v>
+      </c>
+      <c r="O27" s="3">
+        <v>4.6199999999999998E-2</v>
+      </c>
+      <c r="P27" s="3">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="Q27" s="3">
+        <v>5.5599999999999997E-2</v>
+      </c>
+      <c r="R27" s="3">
+        <v>6.3200000000000006E-2</v>
+      </c>
+      <c r="S27" s="3">
+        <v>0.12479999999999999</v>
+      </c>
+      <c r="T27" s="3">
+        <v>5.4100000000000002E-2</v>
+      </c>
+      <c r="U27" s="3">
+        <v>-3.4200000000000001E-2</v>
+      </c>
+      <c r="V27" s="3">
+        <v>0.14560000000000001</v>
+      </c>
+      <c r="W27" s="3">
+        <v>-8.3000000000000001E-3</v>
+      </c>
+      <c r="X27" s="3">
+        <v>0.1159</v>
+      </c>
+      <c r="Y27" s="3">
+        <v>2.01E-2</v>
+      </c>
+      <c r="Z27" s="3">
+        <v>0.12479999999999999</v>
+      </c>
+      <c r="AA27" s="3">
+        <v>5.4100000000000002E-2</v>
+      </c>
+      <c r="AB27" s="3">
+        <v>-3.4200000000000001E-2</v>
+      </c>
+      <c r="AC27" s="3">
+        <v>0.14560000000000001</v>
+      </c>
+      <c r="AD27" s="3">
+        <v>-8.3000000000000001E-3</v>
+      </c>
+      <c r="AE27" s="3">
+        <v>0.1159</v>
+      </c>
+      <c r="AF27" s="3">
+        <v>2.01E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added sagard and mawer
</commit_message>
<xml_diff>
--- a/static/returns/returns.xlsx
+++ b/static/returns/returns.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work Files\ips generator\ips_generator\static\returns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C75FC7-26DA-430C-90EF-0917827AD1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8FFEC3-FEEF-4121-9693-7772F8BE33C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2865" yWindow="3405" windowWidth="38700" windowHeight="15345" xr2:uid="{3B7D21DE-0BB4-48EB-8D25-721726C207C8}"/>
+    <workbookView xWindow="8205" yWindow="3975" windowWidth="38700" windowHeight="15345" xr2:uid="{3B7D21DE-0BB4-48EB-8D25-721726C207C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="80">
   <si>
     <t>Strategy</t>
   </si>
@@ -224,15 +224,9 @@
     <t>Brookfield Private Real Assets Fund</t>
   </si>
   <si>
-    <t>S&amp;P Real Asset Index TR</t>
-  </si>
-  <si>
     <t>Aviso 5-year Bond Ladder (Taxable)</t>
   </si>
   <si>
-    <t>Yield to Maturity Proxy</t>
-  </si>
-  <si>
     <t>Aviso 5-year Bond Ladder (Income)</t>
   </si>
   <si>
@@ -261,6 +255,27 @@
   </si>
   <si>
     <t>2024b</t>
+  </si>
+  <si>
+    <t>Sagard Private Credit Fund</t>
+  </si>
+  <si>
+    <t>Mawer EAFE Large Cap Fund</t>
+  </si>
+  <si>
+    <t>Aviso 5-year Bond Ladder (Income) Bench</t>
+  </si>
+  <si>
+    <t>Aviso 5-year Bond Ladder (Taxable) Bench</t>
+  </si>
+  <si>
+    <t>MSCIWLDNR</t>
+  </si>
+  <si>
+    <t>SPRAUT</t>
+  </si>
+  <si>
+    <t>Morningstar LSTA US Leveraged Loan TR Hdg CAD</t>
   </si>
 </sst>
 </file>
@@ -652,14 +667,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6735C09-F373-4DF4-94E4-3820E8317037}">
-  <dimension ref="A1:AF27"/>
+  <dimension ref="A1:AG29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="94.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -715,28 +730,28 @@
         <v>17</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="V1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="X1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="Z1" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>18</v>
@@ -757,7 +772,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -765,97 +780,100 @@
         <v>25</v>
       </c>
       <c r="C2" s="2">
-        <v>-1.52E-2</v>
+        <v>1.24508333333333E-2</v>
       </c>
       <c r="D2" s="2">
-        <v>-4.4000000000000003E-3</v>
+        <v>1.6722055828822361E-2</v>
       </c>
       <c r="E2" s="2">
-        <v>7.1099999999999997E-2</v>
+        <v>3.2421957557520642E-2</v>
       </c>
       <c r="F2" s="2">
-        <v>7.1099999999999997E-2</v>
+        <v>0.1049618127567562</v>
       </c>
       <c r="G2" s="2">
-        <v>2.23E-2</v>
+        <v>3.8563021682313181E-2</v>
       </c>
       <c r="H2" s="2">
-        <v>4.7899999999999998E-2</v>
+        <v>6.1502983721945848E-2</v>
       </c>
       <c r="I2" s="2">
-        <v>4.6699999999999998E-2</v>
+        <v>4.8305930361838938E-2</v>
       </c>
       <c r="J2" s="2">
-        <v>5.9499999999999997E-2</v>
+        <v>6.0563978398811218E-2</v>
       </c>
       <c r="K2" s="2">
-        <v>-1.2E-2</v>
+        <v>5.4000000000000714E-3</v>
       </c>
       <c r="L2" s="2">
-        <v>1.4999999999999999E-2</v>
+        <v>1.200990175999994E-2</v>
       </c>
       <c r="M2" s="2">
-        <v>0.1022</v>
+        <v>2.430152000000008E-2</v>
       </c>
       <c r="N2" s="2">
-        <v>0.1022</v>
+        <v>0.12811202086357379</v>
       </c>
       <c r="O2" s="2">
-        <v>2.5399999999999999E-2</v>
+        <v>4.4101273556386163E-2</v>
       </c>
       <c r="P2" s="2">
-        <v>4.4299999999999999E-2</v>
+        <v>5.5861172034407103E-2</v>
       </c>
       <c r="Q2" s="2">
-        <v>4.4999999999999998E-2</v>
+        <v>4.6042707792446118E-2</v>
       </c>
       <c r="R2" s="2">
-        <v>5.3900000000000003E-2</v>
+        <v>5.4692512195658072E-2</v>
       </c>
       <c r="S2" s="2">
-        <v>7.1099999999999997E-2</v>
+        <v>7.110857750516808E-2</v>
       </c>
       <c r="T2" s="2">
-        <v>6.9500000000000006E-2</v>
+        <v>6.9503962505472972E-2</v>
       </c>
       <c r="U2" s="2">
-        <v>-6.7400000000000002E-2</v>
+        <v>-6.7351246961500744E-2</v>
       </c>
       <c r="V2" s="2">
-        <v>8.5000000000000006E-2</v>
+        <v>8.5023922266367569E-2</v>
       </c>
       <c r="W2" s="2">
-        <v>8.9800000000000005E-2</v>
+        <v>8.9842946766752751E-2</v>
       </c>
       <c r="X2" s="2">
-        <v>0.1018</v>
+        <v>0.10176585775880009</v>
       </c>
       <c r="Y2" s="2">
-        <v>-2.7000000000000001E-3</v>
+        <v>-2.6719568605251261E-3</v>
       </c>
       <c r="Z2" s="2">
-        <v>0.1022</v>
+        <v>0.1021823224916296</v>
       </c>
       <c r="AA2" s="2">
-        <v>8.77E-2</v>
+        <v>8.7716228179286926E-2</v>
       </c>
       <c r="AB2" s="2">
-        <v>-0.1008</v>
+        <v>-0.1007791321090222</v>
       </c>
       <c r="AC2" s="2">
-        <v>5.45E-2</v>
+        <v>5.4533862712955017E-2</v>
       </c>
       <c r="AD2" s="2">
-        <v>9.2799999999999994E-2</v>
+        <v>9.2753957970583167E-2</v>
       </c>
       <c r="AE2" s="2">
-        <v>0.1169</v>
+        <v>0.1168755683777853</v>
       </c>
       <c r="AF2" s="2">
-        <v>-2.9999999999999997E-4</v>
+        <v>-3.3133518868777578E-4</v>
+      </c>
+      <c r="AG2">
+        <v>36562466.039999999</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -863,97 +881,100 @@
         <v>27</v>
       </c>
       <c r="C3" s="2">
-        <v>2.9999999999999997E-4</v>
+        <v>7.5694677419355649E-3</v>
       </c>
       <c r="D3" s="2">
-        <v>2.5999999999999999E-3</v>
+        <v>1.8621651279313811E-2</v>
       </c>
       <c r="E3" s="2">
-        <v>5.1700000000000003E-2</v>
+        <v>1.832769162855663E-2</v>
       </c>
       <c r="F3" s="2">
-        <v>5.1700000000000003E-2</v>
+        <v>8.0680610327928282E-2</v>
       </c>
       <c r="G3" s="2">
-        <v>1.04E-2</v>
+        <v>2.7230256420633921E-2</v>
       </c>
       <c r="H3" s="2">
-        <v>1.6199999999999999E-2</v>
+        <v>1.7817799621784539E-2</v>
       </c>
       <c r="I3" s="2">
-        <v>1.9099999999999999E-2</v>
+        <v>1.8794602267146129E-2</v>
       </c>
       <c r="J3" s="2">
-        <v>4.3799999999999999E-2</v>
+        <v>4.417193941064701E-2</v>
       </c>
       <c r="K3" s="2">
-        <v>1.5E-3</v>
+        <v>7.3000000000000842E-3</v>
       </c>
       <c r="L3" s="2">
-        <v>2.5999999999999999E-3</v>
+        <v>1.970610826000008E-2</v>
       </c>
       <c r="M3" s="2">
-        <v>5.3400000000000003E-2</v>
+        <v>1.8178840000000029E-2</v>
       </c>
       <c r="N3" s="2">
-        <v>5.3400000000000003E-2</v>
+        <v>8.0432383682738307E-2</v>
       </c>
       <c r="O3" s="2">
-        <v>1.3599999999999999E-2</v>
+        <v>2.9775139913844621E-2</v>
       </c>
       <c r="P3" s="2">
-        <v>1.7000000000000001E-2</v>
+        <v>1.8598628207831199E-2</v>
       </c>
       <c r="Q3" s="2">
-        <v>1.9400000000000001E-2</v>
+        <v>1.9438540178987829E-2</v>
       </c>
       <c r="R3" s="2">
-        <v>4.1099999999999998E-2</v>
+        <v>4.1555062232766733E-2</v>
       </c>
       <c r="S3" s="2">
-        <v>5.1700000000000003E-2</v>
+        <v>5.1696869975270232E-2</v>
       </c>
       <c r="T3" s="2">
-        <v>5.9200000000000003E-2</v>
+        <v>5.9227296447104998E-2</v>
       </c>
       <c r="U3" s="2">
-        <v>-7.4099999999999999E-2</v>
+        <v>-7.4084527114463228E-2</v>
       </c>
       <c r="V3" s="2">
-        <v>-2.0799999999999999E-2</v>
+        <v>-2.07639840561471E-2</v>
       </c>
       <c r="W3" s="2">
-        <v>7.2700000000000001E-2</v>
+        <v>7.2733709335903507E-2</v>
       </c>
       <c r="X3" s="2">
-        <v>4.24E-2</v>
+        <v>4.2417853556049989E-2</v>
       </c>
       <c r="Y3" s="2">
-        <v>1.5100000000000001E-2</v>
+        <v>1.5143026145177931E-2</v>
       </c>
       <c r="Z3" s="2">
-        <v>5.3400000000000003E-2</v>
+        <v>5.3406602437456867E-2</v>
       </c>
       <c r="AA3" s="2">
-        <v>5.4199999999999998E-2</v>
+        <v>5.4237633096663178E-2</v>
       </c>
       <c r="AB3" s="2">
-        <v>-6.2300000000000001E-2</v>
+        <v>-6.2297397020487977E-2</v>
       </c>
       <c r="AC3" s="2">
-        <v>-1.5299999999999999E-2</v>
+        <v>-1.533915638406891E-2</v>
       </c>
       <c r="AD3" s="2">
-        <v>6.1199999999999997E-2</v>
+        <v>6.1174539832829611E-2</v>
       </c>
       <c r="AE3" s="2">
-        <v>4.0300000000000002E-2</v>
+        <v>4.0268031248332781E-2</v>
       </c>
       <c r="AF3" s="2">
-        <v>1.9099999999999999E-2</v>
+        <v>1.9121810314036921E-2</v>
+      </c>
+      <c r="AG3">
+        <v>91652136.950000003</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -961,97 +982,100 @@
         <v>29</v>
       </c>
       <c r="C4" s="2">
-        <v>-1.6899999999999998E-2</v>
+        <v>-1.440096652719669E-2</v>
       </c>
       <c r="D4" s="2">
-        <v>3.73E-2</v>
+        <v>1.491630622523221E-2</v>
       </c>
       <c r="E4" s="2">
-        <v>0.20300000000000001</v>
+        <v>3.2351599341953641E-2</v>
       </c>
       <c r="F4" s="2">
-        <v>0.20300000000000001</v>
+        <v>0.1784816937470011</v>
       </c>
       <c r="G4" s="2">
-        <v>0.12570000000000001</v>
+        <v>0.1345101867807692</v>
       </c>
       <c r="H4" s="2">
-        <v>0.15709999999999999</v>
+        <v>0.18919176413225</v>
       </c>
       <c r="I4" s="2">
-        <v>0.12970000000000001</v>
+        <v>0.12962592369786541</v>
       </c>
       <c r="J4" s="2">
-        <v>9.9299999999999999E-2</v>
+        <v>9.9983608596376117E-2</v>
       </c>
       <c r="K4" s="2">
-        <v>-2.2700000000000001E-2</v>
+        <v>-8.2999999999999741E-3</v>
       </c>
       <c r="L4" s="2">
-        <v>5.3600000000000002E-2</v>
+        <v>7.7621087179999826E-3</v>
       </c>
       <c r="M4" s="2">
-        <v>0.25590000000000002</v>
+        <v>3.1169659999999991E-2</v>
       </c>
       <c r="N4" s="2">
-        <v>0.25590000000000002</v>
+        <v>0.23602978614667311</v>
       </c>
       <c r="O4" s="2">
-        <v>0.1013</v>
+        <v>0.11082720147125411</v>
       </c>
       <c r="P4" s="2">
-        <v>0.13170000000000001</v>
+        <v>0.16652505376055521</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.1109</v>
+        <v>0.11083044738618431</v>
       </c>
       <c r="R4" s="2">
-        <v>6.8400000000000002E-2</v>
+        <v>6.9222481484886966E-2</v>
       </c>
       <c r="S4" s="2">
-        <v>0.20300000000000001</v>
+        <v>0.20300051409891351</v>
       </c>
       <c r="T4" s="2">
-        <v>0.22670000000000001</v>
+        <v>0.22666917874780079</v>
       </c>
       <c r="U4" s="2">
-        <v>-3.3399999999999999E-2</v>
+        <v>-3.3374670046121817E-2</v>
       </c>
       <c r="V4" s="2">
-        <v>0.29480000000000001</v>
+        <v>0.29477003772115862</v>
       </c>
       <c r="W4" s="2">
-        <v>0.1232</v>
+        <v>0.12321388075036779</v>
       </c>
       <c r="X4" s="2">
-        <v>0.1946</v>
+        <v>0.1946031324946251</v>
       </c>
       <c r="Y4" s="2">
-        <v>-2.3E-3</v>
+        <v>-2.283559756047659E-3</v>
       </c>
       <c r="Z4" s="2">
-        <v>0.25590000000000002</v>
+        <v>0.25589403569629132</v>
       </c>
       <c r="AA4" s="2">
-        <v>0.1489</v>
+        <v>0.1488587438947935</v>
       </c>
       <c r="AB4" s="2">
-        <v>-7.4200000000000002E-2</v>
+        <v>-7.4243142523677252E-2</v>
       </c>
       <c r="AC4" s="2">
-        <v>0.27960000000000002</v>
+        <v>0.27962037205920343</v>
       </c>
       <c r="AD4" s="2">
-        <v>8.6199999999999999E-2</v>
+        <v>8.6160849121817984E-2</v>
       </c>
       <c r="AE4" s="2">
-        <v>0.22819999999999999</v>
+        <v>0.22822661859954649</v>
       </c>
       <c r="AF4" s="2">
-        <v>-4.1000000000000002E-2</v>
+        <v>-4.0965727438507897E-2</v>
+      </c>
+      <c r="AG4">
+        <v>194018918.53999999</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -1059,97 +1083,100 @@
         <v>31</v>
       </c>
       <c r="C5" s="2">
-        <v>-1.6E-2</v>
+        <v>7.918828571428671E-3</v>
       </c>
       <c r="D5" s="2">
-        <v>2.3099999999999999E-2</v>
+        <v>1.326329810095417E-2</v>
       </c>
       <c r="E5" s="2">
-        <v>0.1691</v>
+        <v>2.9729444210970572E-2</v>
       </c>
       <c r="F5" s="2">
-        <v>0.1691</v>
+        <v>0.18330786302476729</v>
       </c>
       <c r="G5" s="2">
-        <v>6.7900000000000002E-2</v>
+        <v>8.3112735414645256E-2</v>
       </c>
       <c r="H5" s="2">
-        <v>8.1299999999999997E-2</v>
+        <v>0.1064525704765933</v>
       </c>
       <c r="I5" s="2">
-        <v>6.7299999999999999E-2</v>
+        <v>6.7864542774802139E-2</v>
       </c>
       <c r="J5" s="2">
-        <v>7.7200000000000005E-2</v>
+        <v>7.785440782670916E-2</v>
       </c>
       <c r="K5" s="2">
-        <v>-2.24E-2</v>
+        <v>2.0000000000000022E-3</v>
       </c>
       <c r="L5" s="2">
-        <v>2.2599999999999999E-2</v>
+        <v>4.729768640000076E-3</v>
       </c>
       <c r="M5" s="2">
-        <v>0.1444</v>
+        <v>2.7751400000000089E-2</v>
       </c>
       <c r="N5" s="2">
-        <v>0.1444</v>
+        <v>0.16749776863039581</v>
       </c>
       <c r="O5" s="2">
-        <v>0.05</v>
+        <v>6.0813720199518473E-2</v>
       </c>
       <c r="P5" s="2">
-        <v>7.2300000000000003E-2</v>
+        <v>9.6550005519527415E-2</v>
       </c>
       <c r="Q5" s="2">
-        <v>6.1899999999999997E-2</v>
+        <v>6.2541536792744656E-2</v>
       </c>
       <c r="R5" s="2">
-        <v>7.4099999999999999E-2</v>
+        <v>7.471156024925496E-2</v>
       </c>
       <c r="S5" s="2">
-        <v>0.1691</v>
+        <v>0.16909176936559361</v>
       </c>
       <c r="T5" s="2">
-        <v>0.12330000000000001</v>
+        <v>0.12328855877582499</v>
       </c>
       <c r="U5" s="2">
-        <v>-7.2599999999999998E-2</v>
+        <v>-7.2623009670554461E-2</v>
       </c>
       <c r="V5" s="2">
-        <v>0.1336</v>
+        <v>0.13359880186010689</v>
       </c>
       <c r="W5" s="2">
-        <v>7.0999999999999994E-2</v>
+        <v>7.0964251198278427E-2</v>
       </c>
       <c r="X5" s="2">
-        <v>0.13239999999999999</v>
+        <v>0.1324110955443196</v>
       </c>
       <c r="Y5" s="2">
-        <v>-2.7799999999999998E-2</v>
+        <v>-2.7766693482052299E-2</v>
       </c>
       <c r="Z5" s="2">
-        <v>0.1444</v>
+        <v>0.14435513740520059</v>
       </c>
       <c r="AA5" s="2">
-        <v>9.7299999999999998E-2</v>
+        <v>9.7290450620474145E-2</v>
       </c>
       <c r="AB5" s="2">
-        <v>-7.8100000000000003E-2</v>
+        <v>-7.8060196500178036E-2</v>
       </c>
       <c r="AC5" s="2">
-        <v>0.13519999999999999</v>
+        <v>0.1351871011014274</v>
       </c>
       <c r="AD5" s="2">
-        <v>7.8600000000000003E-2</v>
+        <v>7.8614809902556315E-2</v>
       </c>
       <c r="AE5" s="2">
-        <v>0.1633</v>
+        <v>0.16333273441343341</v>
       </c>
       <c r="AF5" s="2">
-        <v>-4.6600000000000003E-2</v>
+        <v>-4.6556803672422993E-2</v>
+      </c>
+      <c r="AG5">
+        <v>18275998.289999999</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -1157,97 +1184,100 @@
         <v>33</v>
       </c>
       <c r="C6" s="2">
-        <v>-2.1600000000000001E-2</v>
+        <v>5.9103846153845119E-3</v>
       </c>
       <c r="D6" s="2">
-        <v>3.7900000000000003E-2</v>
+        <v>8.8847202734911868E-3</v>
       </c>
       <c r="E6" s="2">
-        <v>0.2465</v>
+        <v>3.1121593962721631E-2</v>
       </c>
       <c r="F6" s="2">
-        <v>0.2465</v>
+        <v>0.24024368450940181</v>
       </c>
       <c r="G6" s="2">
-        <v>0.1099</v>
+        <v>0.11819146980306169</v>
       </c>
       <c r="H6" s="2">
-        <v>0.11650000000000001</v>
+        <v>0.1586984910917506</v>
       </c>
       <c r="I6" s="2">
-        <v>9.0200000000000002E-2</v>
+        <v>9.1123660866985423E-2</v>
       </c>
       <c r="J6" s="2">
-        <v>8.5000000000000006E-2</v>
+        <v>8.5615166196782777E-2</v>
       </c>
       <c r="K6" s="2">
-        <v>-3.27E-2</v>
+        <v>-4.0000000000000044E-3</v>
       </c>
       <c r="L6" s="2">
-        <v>3.7699999999999997E-2</v>
+        <v>-3.041808160000103E-3</v>
       </c>
       <c r="M6" s="2">
-        <v>0.21640000000000001</v>
+        <v>3.0660799999999929E-2</v>
       </c>
       <c r="N6" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.22454925336440401</v>
       </c>
       <c r="O6" s="2">
-        <v>8.6499999999999994E-2</v>
+        <v>8.844086955805297E-2</v>
       </c>
       <c r="P6" s="2">
-        <v>0.11119999999999999</v>
+        <v>0.1534472761844223</v>
       </c>
       <c r="Q6" s="2">
-        <v>8.6699999999999999E-2</v>
+        <v>8.8153012204149617E-2</v>
       </c>
       <c r="R6" s="2">
-        <v>7.46E-2</v>
+        <v>7.5294552309795204E-2</v>
       </c>
       <c r="S6" s="2">
-        <v>0.2465</v>
+        <v>0.2464799745561268</v>
       </c>
       <c r="T6" s="2">
-        <v>0.1482</v>
+        <v>0.1481932347269663</v>
       </c>
       <c r="U6" s="2">
-        <v>-4.4600000000000001E-2</v>
+        <v>-4.4647519966674272E-2</v>
       </c>
       <c r="V6" s="2">
-        <v>0.2286</v>
+        <v>0.22858982038478379</v>
       </c>
       <c r="W6" s="2">
-        <v>3.2599999999999997E-2</v>
+        <v>3.2613190352135168E-2</v>
       </c>
       <c r="X6" s="2">
-        <v>0.1691</v>
+        <v>0.16910836648109909</v>
       </c>
       <c r="Y6" s="2">
-        <v>-6.0699999999999997E-2</v>
+        <v>-6.0702708212991729E-2</v>
       </c>
       <c r="Z6" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.21639791486141899</v>
       </c>
       <c r="AA6" s="2">
-        <v>0.1202</v>
+        <v>0.12021853546487481</v>
       </c>
       <c r="AB6" s="2">
-        <v>-5.8599999999999999E-2</v>
+        <v>-5.861422986020437E-2</v>
       </c>
       <c r="AC6" s="2">
-        <v>0.25090000000000001</v>
+        <v>0.25087973789207202</v>
       </c>
       <c r="AD6" s="2">
-        <v>5.5899999999999998E-2</v>
+        <v>5.5915166451887321E-2</v>
       </c>
       <c r="AE6" s="2">
-        <v>0.2288</v>
+        <v>0.22876839007651761</v>
       </c>
       <c r="AF6" s="2">
-        <v>-8.8900000000000007E-2</v>
+        <v>-8.8861093780151279E-2</v>
+      </c>
+      <c r="AG6">
+        <v>21148869.02</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -1255,97 +1285,100 @@
         <v>35</v>
       </c>
       <c r="C7" s="2">
-        <v>-6.4000000000000003E-3</v>
+        <v>1.2121467391304369E-2</v>
       </c>
       <c r="D7" s="2">
-        <v>1E-4</v>
+        <v>1.8894675461928578E-2</v>
       </c>
       <c r="E7" s="2">
-        <v>4.9799999999999997E-2</v>
+        <v>2.5493836244884219E-2</v>
       </c>
       <c r="F7" s="2">
-        <v>4.9799999999999997E-2</v>
+        <v>9.3862884628607812E-2</v>
       </c>
       <c r="G7" s="2">
-        <v>-4.3E-3</v>
+        <v>2.0995220498161379E-2</v>
       </c>
       <c r="H7" s="2">
-        <v>1.2E-2</v>
+        <v>1.4327082069022451E-2</v>
       </c>
       <c r="I7" s="2">
-        <v>2.1100000000000001E-2</v>
+        <v>2.09171157542416E-2</v>
       </c>
       <c r="J7" s="2">
-        <v>5.2200000000000003E-2</v>
+        <v>5.2740659169707722E-2</v>
       </c>
       <c r="K7" s="2">
-        <v>-6.8999999999999999E-3</v>
+        <v>1.09999999999999E-2</v>
       </c>
       <c r="L7" s="2">
-        <v>-5.0000000000000001E-4</v>
+        <v>1.607238919999987E-2</v>
       </c>
       <c r="M7" s="2">
-        <v>4.2299999999999997E-2</v>
+        <v>2.313199999999993E-2</v>
       </c>
       <c r="N7" s="2">
-        <v>4.2299999999999997E-2</v>
+        <v>8.4867214211104436E-2</v>
       </c>
       <c r="O7" s="2">
-        <v>-7.1999999999999998E-3</v>
+        <v>1.6559852705851918E-2</v>
       </c>
       <c r="P7" s="2">
-        <v>7.1999999999999998E-3</v>
+        <v>9.6988969437727945E-3</v>
       </c>
       <c r="Q7" s="2">
-        <v>1.9400000000000001E-2</v>
+        <v>1.8966073465605641E-2</v>
       </c>
       <c r="R7" s="2">
-        <v>5.0599999999999999E-2</v>
+        <v>5.1124428236377861E-2</v>
       </c>
       <c r="S7" s="2">
-        <v>4.9799999999999997E-2</v>
+        <v>4.9758392035209147E-2</v>
       </c>
       <c r="T7" s="2">
-        <v>7.46E-2</v>
+        <v>7.4649345331067485E-2</v>
       </c>
       <c r="U7" s="2">
-        <v>-0.125</v>
+        <v>-0.12497102831907179</v>
       </c>
       <c r="V7" s="2">
-        <v>-2.52E-2</v>
+        <v>-2.5217556612129769E-2</v>
       </c>
       <c r="W7" s="2">
-        <v>0.10290000000000001</v>
+        <v>0.10285331526718069</v>
       </c>
       <c r="X7" s="2">
-        <v>6.5000000000000002E-2</v>
+        <v>6.5038215096127949E-2</v>
       </c>
       <c r="Y7" s="2">
-        <v>1.24E-2</v>
+        <v>1.2437482995890649E-2</v>
       </c>
       <c r="Z7" s="2">
-        <v>4.2299999999999997E-2</v>
+        <v>4.2257028382391093E-2</v>
       </c>
       <c r="AA7" s="2">
-        <v>6.3100000000000003E-2</v>
+        <v>6.3062276236460102E-2</v>
       </c>
       <c r="AB7" s="2">
-        <v>-0.1169</v>
+        <v>-0.11689077106871799</v>
       </c>
       <c r="AC7" s="2">
-        <v>-2.5399999999999999E-2</v>
+        <v>-2.5394156876443419E-2</v>
       </c>
       <c r="AD7" s="2">
-        <v>8.6800000000000002E-2</v>
+        <v>8.6757289789715752E-2</v>
       </c>
       <c r="AE7" s="2">
-        <v>6.8699999999999997E-2</v>
+        <v>6.8712084440473165E-2</v>
       </c>
       <c r="AF7" s="2">
-        <v>1.41E-2</v>
+        <v>1.4079379818825901E-2</v>
+      </c>
+      <c r="AG7">
+        <v>91233383.430000007</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -1353,97 +1386,100 @@
         <v>37</v>
       </c>
       <c r="C8" s="2">
-        <v>7.4000000000000003E-3</v>
+        <v>-5.3746141732283759E-3</v>
       </c>
       <c r="D8" s="2">
-        <v>4.7800000000000002E-2</v>
+        <v>4.5854165693122402E-2</v>
       </c>
       <c r="E8" s="2">
-        <v>0.2596</v>
+        <v>3.8168900316720933E-2</v>
       </c>
       <c r="F8" s="2">
-        <v>0.2596</v>
+        <v>0.21379324138002501</v>
       </c>
       <c r="G8" s="2">
-        <v>0.1057</v>
+        <v>0.13632166281808281</v>
       </c>
       <c r="H8" s="2">
-        <v>0.13189999999999999</v>
+        <v>0.15509314804414381</v>
       </c>
       <c r="I8" s="2">
-        <v>0.1172</v>
+        <v>0.11435879204735989</v>
       </c>
       <c r="J8" s="2">
-        <v>0.1052</v>
+        <v>0.1062437853248233</v>
       </c>
       <c r="K8" s="2">
-        <v>4.0000000000000002E-4</v>
+        <v>-1.2499999999999961E-2</v>
       </c>
       <c r="L8" s="2">
-        <v>6.2899999999999998E-2</v>
+        <v>2.9880537499999971E-2</v>
       </c>
       <c r="M8" s="2">
-        <v>0.29430000000000001</v>
+        <v>2.9468749999999929E-2</v>
       </c>
       <c r="N8" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.2279335112320855</v>
       </c>
       <c r="O8" s="2">
-        <v>0.114</v>
+        <v>0.1406458000440951</v>
       </c>
       <c r="P8" s="2">
-        <v>0.13700000000000001</v>
+        <v>0.1663213492098834</v>
       </c>
       <c r="Q8" s="2">
-        <v>0.12770000000000001</v>
+        <v>0.12248757151155699</v>
       </c>
       <c r="R8" s="2">
-        <v>9.3299999999999994E-2</v>
+        <v>9.4006958248271877E-2</v>
       </c>
       <c r="S8" s="2">
-        <v>0.2596</v>
+        <v>0.25956354944849203</v>
       </c>
       <c r="T8" s="2">
-        <v>0.1754</v>
+        <v>0.1753993264425078</v>
       </c>
       <c r="U8" s="2">
-        <v>-8.6900000000000005E-2</v>
+        <v>-8.6883515521638199E-2</v>
       </c>
       <c r="V8" s="2">
-        <v>0.26769999999999999</v>
+        <v>0.26766545352246007</v>
       </c>
       <c r="W8" s="2">
-        <v>8.4199999999999997E-2</v>
+        <v>8.4249303506370277E-2</v>
       </c>
       <c r="X8" s="2">
-        <v>0.19639999999999999</v>
+        <v>0.19638981733600039</v>
       </c>
       <c r="Y8" s="2">
-        <v>-5.0000000000000001E-3</v>
+        <v>-4.9599140354200646E-3</v>
       </c>
       <c r="Z8" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.29426365037508218</v>
       </c>
       <c r="AA8" s="2">
-        <v>0.2102</v>
+        <v>0.21016918258785361</v>
       </c>
       <c r="AB8" s="2">
-        <v>-0.11749999999999999</v>
+        <v>-0.1174573603921328</v>
       </c>
       <c r="AC8" s="2">
-        <v>0.21310000000000001</v>
+        <v>0.21310109733026381</v>
       </c>
       <c r="AD8" s="2">
-        <v>0.13320000000000001</v>
+        <v>0.13322710348184111</v>
       </c>
       <c r="AE8" s="2">
-        <v>0.21909999999999999</v>
+        <v>0.21910476774026419</v>
       </c>
       <c r="AF8" s="2">
-        <v>5.9999999999999995E-4</v>
+        <v>6.3113667818059938E-4</v>
+      </c>
+      <c r="AG8">
+        <v>122618881.38</v>
       </c>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -1451,97 +1487,100 @@
         <v>37</v>
       </c>
       <c r="C9" s="2">
-        <v>4.4999999999999997E-3</v>
+        <v>-7.6082558139535239E-3</v>
       </c>
       <c r="D9" s="2">
-        <v>4.7699999999999999E-2</v>
+        <v>4.13274011843483E-2</v>
       </c>
       <c r="E9" s="2">
-        <v>0.26279999999999998</v>
+        <v>3.6635567871450947E-2</v>
       </c>
       <c r="F9" s="2">
-        <v>0.26279999999999998</v>
+        <v>0.21448341747325911</v>
       </c>
       <c r="G9" s="2">
-        <v>0.10299999999999999</v>
+        <v>0.13775310599180979</v>
       </c>
       <c r="H9" s="2">
-        <v>0.1384</v>
+        <v>0.16183008748527139</v>
       </c>
       <c r="I9" s="2">
-        <v>0.121</v>
+        <v>0.1175711466571818</v>
       </c>
       <c r="J9" s="2">
-        <v>8.9599999999999999E-2</v>
+        <v>9.0977203684160513E-2</v>
       </c>
       <c r="K9" s="2">
-        <v>4.0000000000000002E-4</v>
+        <v>-1.2499999999999961E-2</v>
       </c>
       <c r="L9" s="2">
-        <v>6.2899999999999998E-2</v>
+        <v>2.9880537499999971E-2</v>
       </c>
       <c r="M9" s="2">
-        <v>0.29430000000000001</v>
+        <v>2.9468749999999929E-2</v>
       </c>
       <c r="N9" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.2279335112320855</v>
       </c>
       <c r="O9" s="2">
-        <v>0.114</v>
+        <v>0.1406458000440951</v>
       </c>
       <c r="P9" s="2">
-        <v>0.13700000000000001</v>
+        <v>0.1663213492098834</v>
       </c>
       <c r="Q9" s="2">
-        <v>0.12770000000000001</v>
+        <v>0.12248757151155699</v>
       </c>
       <c r="R9" s="2">
-        <v>0.1003</v>
+        <v>0.1011815742271851</v>
       </c>
       <c r="S9" s="2">
-        <v>0.26279999999999998</v>
+        <v>0.26275886187340619</v>
       </c>
       <c r="T9" s="2">
-        <v>0.19209999999999999</v>
+        <v>0.19210350219382619</v>
       </c>
       <c r="U9" s="2">
-        <v>-0.1086</v>
+        <v>-0.1086485740791715</v>
       </c>
       <c r="V9" s="2">
-        <v>0.31929999999999997</v>
+        <v>0.31928245119478338</v>
       </c>
       <c r="W9" s="2">
-        <v>0.08</v>
+        <v>7.9992473769204819E-2</v>
       </c>
       <c r="X9" s="2">
-        <v>0.2155</v>
+        <v>0.2154545270790329</v>
       </c>
       <c r="Y9" s="2">
-        <v>8.6E-3</v>
+        <v>8.5866506209266724E-3</v>
       </c>
       <c r="Z9" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.29426365037508218</v>
       </c>
       <c r="AA9" s="2">
-        <v>0.2102</v>
+        <v>0.21016918258785361</v>
       </c>
       <c r="AB9" s="2">
-        <v>-0.11749999999999999</v>
+        <v>-0.1174573603921328</v>
       </c>
       <c r="AC9" s="2">
-        <v>0.21310000000000001</v>
+        <v>0.21310109733026381</v>
       </c>
       <c r="AD9" s="2">
-        <v>0.13320000000000001</v>
+        <v>0.13322710348184111</v>
       </c>
       <c r="AE9" s="2">
-        <v>0.21909999999999999</v>
+        <v>0.21910476774026419</v>
       </c>
       <c r="AF9" s="2">
-        <v>5.9999999999999995E-4</v>
+        <v>6.3113667818059938E-4</v>
+      </c>
+      <c r="AG9">
+        <v>39805919.340000004</v>
       </c>
     </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -1549,97 +1588,100 @@
         <v>40</v>
       </c>
       <c r="C10" s="2">
-        <v>-3.56E-2</v>
+        <v>1.8945222222222169E-2</v>
       </c>
       <c r="D10" s="2">
-        <v>-1.0800000000000001E-2</v>
+        <v>7.2532924185209069E-3</v>
       </c>
       <c r="E10" s="2">
-        <v>0.1331</v>
+        <v>4.4392950117654761E-2</v>
       </c>
       <c r="F10" s="2">
-        <v>0.1331</v>
+        <v>0.18009142345083079</v>
       </c>
       <c r="G10" s="2">
-        <v>9.3799999999999994E-2</v>
+        <v>8.679407272750117E-2</v>
       </c>
       <c r="H10" s="2">
-        <v>9.9599999999999994E-2</v>
+        <v>0.14945988183847941</v>
       </c>
       <c r="I10" s="2">
-        <v>7.5600000000000001E-2</v>
+        <v>7.8806861055847222E-2</v>
       </c>
       <c r="J10" s="2">
-        <v>0.1118</v>
+        <v>0.11308402972963801</v>
       </c>
       <c r="K10" s="2">
-        <v>-3.3399999999999999E-2</v>
+        <v>7.3000000000000842E-3</v>
       </c>
       <c r="L10" s="2">
-        <v>7.7000000000000002E-3</v>
+        <v>-9.5969337039998326E-3</v>
       </c>
       <c r="M10" s="2">
-        <v>0.157</v>
+        <v>2.4625560000000268E-2</v>
       </c>
       <c r="N10" s="2">
-        <v>0.157</v>
+        <v>0.17748268133895739</v>
       </c>
       <c r="O10" s="2">
-        <v>7.9600000000000004E-2</v>
+        <v>6.2201389485577741E-2</v>
       </c>
       <c r="P10" s="2">
-        <v>9.6600000000000005E-2</v>
+        <v>0.15014573708926321</v>
       </c>
       <c r="Q10" s="2">
-        <v>7.7200000000000005E-2</v>
+        <v>7.9416698848171485E-2</v>
       </c>
       <c r="R10" s="2">
-        <v>0.106</v>
+        <v>0.1064120381222424</v>
       </c>
       <c r="S10" s="2">
-        <v>0.1331</v>
+        <v>0.13308185228320671</v>
       </c>
       <c r="T10" s="2">
-        <v>8.8700000000000001E-2</v>
+        <v>8.8744440171499184E-2</v>
       </c>
       <c r="U10" s="2">
-        <v>6.08E-2</v>
+        <v>6.0759705977495797E-2</v>
       </c>
       <c r="V10" s="2">
-        <v>0.30959999999999999</v>
+        <v>0.30956324056409512</v>
       </c>
       <c r="W10" s="2">
-        <v>-6.2E-2</v>
+        <v>-6.2025403848959597E-2</v>
       </c>
       <c r="X10" s="2">
-        <v>0.20830000000000001</v>
+        <v>0.2082705208707534</v>
       </c>
       <c r="Y10" s="2">
-        <v>-0.1009</v>
+        <v>-0.1009024960682712</v>
       </c>
       <c r="Z10" s="2">
-        <v>0.157</v>
+        <v>0.1570007856603988</v>
       </c>
       <c r="AA10" s="2">
-        <v>8.0500000000000002E-2</v>
+        <v>8.050188529371205E-2</v>
       </c>
       <c r="AB10" s="2">
-        <v>6.4000000000000003E-3</v>
+        <v>6.431543794565231E-3</v>
       </c>
       <c r="AC10" s="2">
-        <v>0.36099999999999999</v>
+        <v>0.36103956698877088</v>
       </c>
       <c r="AD10" s="2">
-        <v>-7.3899999999999993E-2</v>
+        <v>-7.3860041217950645E-2</v>
       </c>
       <c r="AE10" s="2">
-        <v>0.2581</v>
+        <v>0.25812480061619558</v>
       </c>
       <c r="AF10" s="2">
-        <v>-0.1077</v>
+        <v>-0.107731401591228</v>
+      </c>
+      <c r="AG10">
+        <v>12875041.279999999</v>
       </c>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -1647,97 +1689,100 @@
         <v>42</v>
       </c>
       <c r="C11" s="2">
-        <v>-1.3100000000000001E-2</v>
+        <v>-1.3420137254901991E-2</v>
       </c>
       <c r="D11" s="2">
-        <v>4.7699999999999999E-2</v>
+        <v>8.140361089503223E-3</v>
       </c>
       <c r="E11" s="2">
-        <v>0.1832</v>
+        <v>2.153940941985022E-2</v>
       </c>
       <c r="F11" s="2">
-        <v>0.1832</v>
+        <v>0.1600602187976301</v>
       </c>
       <c r="G11" s="2">
-        <v>6.5000000000000002E-2</v>
+        <v>9.0287993205319772E-2</v>
       </c>
       <c r="H11" s="2">
-        <v>8.5800000000000001E-2</v>
+        <v>0.10381088748291489</v>
       </c>
       <c r="I11" s="2">
-        <v>7.9500000000000001E-2</v>
+        <v>7.7911945543049477E-2</v>
       </c>
       <c r="J11" s="2">
-        <v>7.8200000000000006E-2</v>
+        <v>7.8496357094812064E-2</v>
       </c>
       <c r="K11" s="2">
-        <v>-1.0999999999999999E-2</v>
+        <v>-9.9999999999988987E-5</v>
       </c>
       <c r="L11" s="2">
-        <v>3.15E-2</v>
+        <v>1.204138573999991E-2</v>
       </c>
       <c r="M11" s="2">
-        <v>0.1605</v>
+        <v>2.3297660000000109E-2</v>
       </c>
       <c r="N11" s="2">
-        <v>0.1605</v>
+        <v>0.16155697124099541</v>
       </c>
       <c r="O11" s="2">
-        <v>5.2400000000000002E-2</v>
+        <v>7.0034058988779124E-2</v>
       </c>
       <c r="P11" s="2">
-        <v>7.46E-2</v>
+        <v>9.0777320025655195E-2</v>
       </c>
       <c r="Q11" s="2">
-        <v>7.0999999999999994E-2</v>
+        <v>6.9785817526893723E-2</v>
       </c>
       <c r="R11" s="2">
-        <v>7.0900000000000005E-2</v>
+        <v>7.1317974567514097E-2</v>
       </c>
       <c r="S11" s="2">
-        <v>0.1832</v>
+        <v>0.18322548414762951</v>
       </c>
       <c r="T11" s="2">
-        <v>0.17330000000000001</v>
+        <v>0.17330481297705999</v>
       </c>
       <c r="U11" s="2">
-        <v>-0.13</v>
+        <v>-0.12996610793626931</v>
       </c>
       <c r="V11" s="2">
-        <v>0.16259999999999999</v>
+        <v>0.16260778923755589</v>
       </c>
       <c r="W11" s="2">
-        <v>7.4899999999999994E-2</v>
+        <v>7.4865762310155848E-2</v>
       </c>
       <c r="X11" s="2">
-        <v>0.1263</v>
+        <v>0.12625265700684721</v>
       </c>
       <c r="Y11" s="2">
-        <v>1.7299999999999999E-2</v>
+        <v>1.7279870544707251E-2</v>
       </c>
       <c r="Z11" s="2">
-        <v>0.1605</v>
+        <v>0.16047266730424201</v>
       </c>
       <c r="AA11" s="2">
-        <v>0.1148</v>
+        <v>0.1147928272931185</v>
       </c>
       <c r="AB11" s="2">
-        <v>-9.9000000000000005E-2</v>
+        <v>-9.9044415340767022E-2</v>
       </c>
       <c r="AC11" s="2">
-        <v>0.1129</v>
+        <v>0.112867795062521</v>
       </c>
       <c r="AD11" s="2">
-        <v>0.1046</v>
+        <v>0.1046288022437831</v>
       </c>
       <c r="AE11" s="2">
-        <v>0.152</v>
+        <v>0.15197488384327329</v>
       </c>
       <c r="AF11" s="2">
-        <v>-6.1999999999999998E-3</v>
+        <v>-6.1622847520066406E-3</v>
+      </c>
+      <c r="AG11">
+        <v>106782884.31999999</v>
       </c>
     </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -1745,97 +1790,100 @@
         <v>44</v>
       </c>
       <c r="C12" s="2">
-        <v>-1.7999999999999999E-2</v>
+        <v>-2.7202454545454561E-2</v>
       </c>
       <c r="D12" s="2">
-        <v>7.5999999999999998E-2</v>
+        <v>4.139584885668901E-3</v>
       </c>
       <c r="E12" s="2">
-        <v>0.28820000000000001</v>
+        <v>2.2532067587102581E-2</v>
       </c>
       <c r="F12" s="2">
-        <v>0.28820000000000001</v>
+        <v>0.21482190052553299</v>
       </c>
       <c r="G12" s="2">
-        <v>0.11600000000000001</v>
+        <v>0.14321177678706659</v>
       </c>
       <c r="H12" s="2">
-        <v>0.13489999999999999</v>
+        <v>0.16398219118923299</v>
       </c>
       <c r="I12" s="2">
-        <v>0.1144</v>
+        <v>0.11228653030534549</v>
       </c>
       <c r="J12" s="2">
-        <v>0.10249999999999999</v>
+        <v>0.1027610864985045</v>
       </c>
       <c r="K12" s="2">
-        <v>-1.4999999999999999E-2</v>
+        <v>-1.1199999999999989E-2</v>
       </c>
       <c r="L12" s="2">
-        <v>6.3899999999999998E-2</v>
+        <v>7.9594831999998394E-3</v>
       </c>
       <c r="M12" s="2">
-        <v>0.28960000000000002</v>
+        <v>2.3309119999999961E-2</v>
       </c>
       <c r="N12" s="2">
-        <v>0.28960000000000002</v>
+        <v>0.242032551733292</v>
       </c>
       <c r="O12" s="2">
-        <v>0.1144</v>
+        <v>0.1252717903859055</v>
       </c>
       <c r="P12" s="2">
-        <v>0.1414</v>
+        <v>0.17458595810543279</v>
       </c>
       <c r="Q12" s="2">
-        <v>0.1222</v>
+        <v>0.1200798665158682</v>
       </c>
       <c r="R12" s="2">
-        <v>9.0200000000000002E-2</v>
+        <v>9.0552237365185695E-2</v>
       </c>
       <c r="S12" s="2">
-        <v>0.28820000000000001</v>
+        <v>0.28821327176199668</v>
       </c>
       <c r="T12" s="2">
-        <v>0.2409</v>
+        <v>0.24089152985559159</v>
       </c>
       <c r="U12" s="2">
-        <v>-0.13059999999999999</v>
+        <v>-0.13059519460896579</v>
       </c>
       <c r="V12" s="2">
-        <v>0.25240000000000001</v>
+        <v>0.25237616768120769</v>
       </c>
       <c r="W12" s="2">
-        <v>8.1600000000000006E-2</v>
+        <v>8.1569070295306689E-2</v>
       </c>
       <c r="X12" s="2">
-        <v>0.17150000000000001</v>
+        <v>0.1715094882487038</v>
       </c>
       <c r="Y12" s="2">
-        <v>9.1999999999999998E-3</v>
+        <v>9.1529806240275846E-3</v>
       </c>
       <c r="Z12" s="2">
-        <v>0.28960000000000002</v>
+        <v>0.28958074617418311</v>
       </c>
       <c r="AA12" s="2">
-        <v>0.1714</v>
+        <v>0.1713694717429799</v>
       </c>
       <c r="AB12" s="2">
-        <v>-8.3900000000000002E-2</v>
+        <v>-8.3909329309362457E-2</v>
       </c>
       <c r="AC12" s="2">
-        <v>0.26400000000000001</v>
+        <v>0.26398989980912058</v>
       </c>
       <c r="AD12" s="2">
-        <v>0.1076</v>
+        <v>0.1075575934363073</v>
       </c>
       <c r="AE12" s="2">
-        <v>0.23880000000000001</v>
+        <v>0.23879323438722061</v>
       </c>
       <c r="AF12" s="2">
-        <v>-2.4400000000000002E-2</v>
+        <v>-2.4421037083545372E-2</v>
+      </c>
+      <c r="AG12">
+        <v>37499681.399999999</v>
       </c>
     </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -1843,97 +1891,100 @@
         <v>46</v>
       </c>
       <c r="C13" s="2">
-        <v>-1.04E-2</v>
+        <v>-4.4192049180327819E-2</v>
       </c>
       <c r="D13" s="2">
-        <v>8.0600000000000005E-2</v>
+        <v>-2.6737882786119771E-3</v>
       </c>
       <c r="E13" s="2">
-        <v>0.2737</v>
+        <v>7.8171064540912827E-3</v>
       </c>
       <c r="F13" s="2">
-        <v>0.2737</v>
+        <v>0.18381795671660581</v>
       </c>
       <c r="G13" s="2">
-        <v>0.10440000000000001</v>
+        <v>0.1265569932867503</v>
       </c>
       <c r="H13" s="2">
-        <v>0.16619999999999999</v>
+        <v>0.18147028888424499</v>
       </c>
       <c r="I13" s="2">
-        <v>0.1515</v>
+        <v>0.14516575586870251</v>
       </c>
       <c r="J13" s="2">
-        <v>0.10050000000000001</v>
+        <v>0.1000872749936903</v>
       </c>
       <c r="K13" s="2">
-        <v>2.7000000000000001E-3</v>
+        <v>-1.8299999999999979E-2</v>
       </c>
       <c r="L13" s="2">
-        <v>9.0300000000000005E-2</v>
+        <v>1.8802860649999701E-2</v>
       </c>
       <c r="M13" s="2">
-        <v>0.36380000000000001</v>
+        <v>1.605949999999989E-2</v>
       </c>
       <c r="N13" s="2">
-        <v>0.36380000000000001</v>
+        <v>0.25764938941815968</v>
       </c>
       <c r="O13" s="2">
-        <v>0.13730000000000001</v>
+        <v>0.1583162539418059</v>
       </c>
       <c r="P13" s="2">
-        <v>0.1681</v>
+        <v>0.19217134054854479</v>
       </c>
       <c r="Q13" s="2">
-        <v>0.1552</v>
+        <v>0.14946663466863039</v>
       </c>
       <c r="R13" s="2">
-        <v>7.5499999999999998E-2</v>
+        <v>7.5641001525709406E-2</v>
       </c>
       <c r="S13" s="2">
-        <v>0.2737</v>
+        <v>0.27366522335215349</v>
       </c>
       <c r="T13" s="2">
-        <v>0.25430000000000003</v>
+        <v>0.25428923880210452</v>
       </c>
       <c r="U13" s="2">
-        <v>-0.15690000000000001</v>
+        <v>-0.15689063861803829</v>
       </c>
       <c r="V13" s="2">
-        <v>0.27160000000000001</v>
+        <v>0.27161910953713958</v>
       </c>
       <c r="W13" s="2">
-        <v>0.25950000000000001</v>
+        <v>0.2595160966611858</v>
       </c>
       <c r="X13" s="2">
-        <v>0.27379999999999999</v>
+        <v>0.27375498705892748</v>
       </c>
       <c r="Y13" s="2">
-        <v>5.3499999999999999E-2</v>
+        <v>5.3456934933305167E-2</v>
       </c>
       <c r="Z13" s="2">
-        <v>0.36380000000000001</v>
+        <v>0.36378001862312792</v>
       </c>
       <c r="AA13" s="2">
-        <v>0.22800000000000001</v>
+        <v>0.22802772224653481</v>
       </c>
       <c r="AB13" s="2">
-        <v>-0.1215</v>
+        <v>-0.12152410109853</v>
       </c>
       <c r="AC13" s="2">
-        <v>0.27610000000000001</v>
+        <v>0.2761454551589928</v>
       </c>
       <c r="AD13" s="2">
-        <v>0.1583</v>
+        <v>0.15829193424188981</v>
       </c>
       <c r="AE13" s="2">
-        <v>0.24840000000000001</v>
+        <v>0.24838940926861031</v>
       </c>
       <c r="AF13" s="2">
-        <v>4.2299999999999997E-2</v>
+        <v>4.2275010225730332E-2</v>
+      </c>
+      <c r="AG13">
+        <v>63175036.729999997</v>
       </c>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>47</v>
       </c>
@@ -1941,97 +1992,100 @@
         <v>33</v>
       </c>
       <c r="C14" s="2">
-        <v>-2.1600000000000001E-2</v>
+        <v>-4.7083781512604617E-3</v>
       </c>
       <c r="D14" s="2">
-        <v>1.9300000000000001E-2</v>
+        <v>-8.3803026289983595E-3</v>
       </c>
       <c r="E14" s="2">
-        <v>0.19389999999999999</v>
+        <v>1.346037181810167E-2</v>
       </c>
       <c r="F14" s="2">
-        <v>0.19389999999999999</v>
+        <v>0.15895056324829479</v>
       </c>
       <c r="G14" s="2">
-        <v>9.8100000000000007E-2</v>
+        <v>8.9560796014035438E-2</v>
       </c>
       <c r="H14" s="2">
-        <v>0.1096</v>
+        <v>0.15131163075430359</v>
       </c>
       <c r="I14" s="2">
-        <v>7.9200000000000007E-2</v>
+        <v>7.9066382825266457E-2</v>
       </c>
       <c r="J14" s="2">
-        <v>0.1179</v>
+        <v>0.117651463165463</v>
       </c>
       <c r="K14" s="2">
-        <v>-3.27E-2</v>
+        <v>-4.0000000000000044E-3</v>
       </c>
       <c r="L14" s="2">
-        <v>3.7699999999999997E-2</v>
+        <v>-3.041808160000103E-3</v>
       </c>
       <c r="M14" s="2">
-        <v>0.21640000000000001</v>
+        <v>3.0660799999999929E-2</v>
       </c>
       <c r="N14" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.22454925336440401</v>
       </c>
       <c r="O14" s="2">
-        <v>8.6499999999999994E-2</v>
+        <v>8.844086955805297E-2</v>
       </c>
       <c r="P14" s="2">
-        <v>0.11119999999999999</v>
+        <v>0.1534472761844223</v>
       </c>
       <c r="Q14" s="2">
-        <v>8.6699999999999999E-2</v>
+        <v>8.8153012204149617E-2</v>
       </c>
       <c r="R14" s="2">
-        <v>8.0600000000000005E-2</v>
+        <v>8.1277551446557572E-2</v>
       </c>
       <c r="S14" s="2">
-        <v>0.19389999999999999</v>
+        <v>0.19391940521041101</v>
       </c>
       <c r="T14" s="2">
-        <v>8.2299999999999998E-2</v>
+        <v>8.2265292556218395E-2</v>
       </c>
       <c r="U14" s="2">
-        <v>2.4899999999999999E-2</v>
+        <v>2.4852794580773718E-2</v>
       </c>
       <c r="V14" s="2">
-        <v>0.2828</v>
+        <v>0.28277174917337572</v>
       </c>
       <c r="W14" s="2">
-        <v>-0.01</v>
+        <v>-9.987112125977915E-3</v>
       </c>
       <c r="X14" s="2">
-        <v>0.2046</v>
+        <v>0.20463900163792559</v>
       </c>
       <c r="Y14" s="2">
-        <v>-0.11310000000000001</v>
+        <v>-0.1130749971911198</v>
       </c>
       <c r="Z14" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.21639791486141899</v>
       </c>
       <c r="AA14" s="2">
-        <v>0.1202</v>
+        <v>0.12021853546487481</v>
       </c>
       <c r="AB14" s="2">
-        <v>-5.8599999999999999E-2</v>
+        <v>-5.861422986020437E-2</v>
       </c>
       <c r="AC14" s="2">
-        <v>0.25090000000000001</v>
+        <v>0.25087973789207202</v>
       </c>
       <c r="AD14" s="2">
-        <v>5.5899999999999998E-2</v>
+        <v>5.5915166451887321E-2</v>
       </c>
       <c r="AE14" s="2">
-        <v>0.2288</v>
+        <v>0.22876839007651761</v>
       </c>
       <c r="AF14" s="2">
-        <v>-8.8900000000000007E-2</v>
+        <v>-8.8861093780151279E-2</v>
+      </c>
+      <c r="AG14">
+        <v>100366932.59</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>48</v>
       </c>
@@ -2039,97 +2093,100 @@
         <v>49</v>
       </c>
       <c r="C15" s="2">
-        <v>-1.52E-2</v>
+        <v>-2.7122199999999989E-2</v>
       </c>
       <c r="D15" s="2">
-        <v>1.0500000000000001E-2</v>
+        <v>1.3133811032997929E-2</v>
       </c>
       <c r="E15" s="2">
-        <v>0.14549999999999999</v>
+        <v>2.877356976509016E-2</v>
       </c>
       <c r="F15" s="2">
-        <v>0.14549999999999999</v>
+        <v>0.14963819388483299</v>
       </c>
       <c r="G15" s="2">
-        <v>9.2499999999999999E-2</v>
+        <v>9.5605664391316791E-2</v>
       </c>
       <c r="H15" s="2">
-        <v>0.1135</v>
+        <v>0.17091819024024679</v>
       </c>
       <c r="I15" s="2">
-        <v>8.6800000000000002E-2</v>
+        <v>8.983680290657281E-2</v>
       </c>
       <c r="J15" s="2">
-        <v>0.1123</v>
+        <v>0.1127018313800365</v>
       </c>
       <c r="K15" s="2">
-        <v>-3.3000000000000002E-2</v>
+        <v>-2.270000000000005E-2</v>
       </c>
       <c r="L15" s="2">
-        <v>6.7999999999999996E-3</v>
+        <v>-4.8808080850000102E-2</v>
       </c>
       <c r="M15" s="2">
-        <v>0.17910000000000001</v>
+        <v>-1.63475500000001E-2</v>
       </c>
       <c r="N15" s="2">
-        <v>0.17910000000000001</v>
+        <v>0.16415145540221809</v>
       </c>
       <c r="O15" s="2">
-        <v>3.8699999999999998E-2</v>
+        <v>1.7771351911434641E-2</v>
       </c>
       <c r="P15" s="2">
-        <v>9.8599999999999993E-2</v>
+        <v>0.16268018594929259</v>
       </c>
       <c r="Q15" s="2">
-        <v>6.8500000000000005E-2</v>
+        <v>6.6691636391552844E-2</v>
       </c>
       <c r="R15" s="2">
-        <v>6.2600000000000003E-2</v>
+        <v>6.1561346956535479E-2</v>
       </c>
       <c r="S15" s="2">
-        <v>0.14549999999999999</v>
+        <v>0.1454564677544905</v>
       </c>
       <c r="T15" s="2">
-        <v>0.13159999999999999</v>
+        <v>0.13163604439679649</v>
       </c>
       <c r="U15" s="2">
-        <v>6.0000000000000001E-3</v>
+        <v>6.004942311459649E-3</v>
       </c>
       <c r="V15" s="2">
-        <v>0.2596</v>
+        <v>0.25963045708737781</v>
       </c>
       <c r="W15" s="2">
-        <v>4.2299999999999997E-2</v>
+        <v>4.2266551135459629E-2</v>
       </c>
       <c r="X15" s="2">
-        <v>0.1744</v>
+        <v>0.174356775690232</v>
       </c>
       <c r="Y15" s="2">
-        <v>-9.0999999999999998E-2</v>
+        <v>-9.1042596803016851E-2</v>
       </c>
       <c r="Z15" s="2">
-        <v>0.17910000000000001</v>
+        <v>0.17911981515140821</v>
       </c>
       <c r="AA15" s="2">
-        <v>4.7E-2</v>
+        <v>4.7003170409684943E-2</v>
       </c>
       <c r="AB15" s="2">
-        <v>-9.2200000000000004E-2</v>
+        <v>-9.2181445783686145E-2</v>
       </c>
       <c r="AC15" s="2">
-        <v>0.24790000000000001</v>
+        <v>0.2479183845762456</v>
       </c>
       <c r="AD15" s="2">
-        <v>0.14419999999999999</v>
+        <v>0.14422856360136599</v>
       </c>
       <c r="AE15" s="2">
-        <v>0.192</v>
+        <v>0.19203163120775571</v>
       </c>
       <c r="AF15" s="2">
-        <v>-0.1817</v>
+        <v>-0.18167452986828991</v>
+      </c>
+      <c r="AG15">
+        <v>15122269.26</v>
       </c>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>50</v>
       </c>
@@ -2137,97 +2194,100 @@
         <v>33</v>
       </c>
       <c r="C16" s="2">
-        <v>-3.1899999999999998E-2</v>
+        <v>-1.0710000000000001E-2</v>
       </c>
       <c r="D16" s="2">
-        <v>1.3599999999999999E-2</v>
+        <v>-2.350010568781935E-2</v>
       </c>
       <c r="E16" s="2">
-        <v>0.17899999999999999</v>
+        <v>8.6735546859999513E-3</v>
       </c>
       <c r="F16" s="2">
-        <v>0.17899999999999999</v>
+        <v>0.16476171868558559</v>
       </c>
       <c r="G16" s="2">
-        <v>9.6799999999999997E-2</v>
+        <v>8.1191072392124308E-2</v>
       </c>
       <c r="H16" s="2">
-        <v>0.1206</v>
+        <v>0.16115318539571</v>
       </c>
       <c r="I16" s="2">
-        <v>9.5299999999999996E-2</v>
+        <v>9.5629547620493138E-2</v>
       </c>
       <c r="J16" s="2">
-        <v>9.7199999999999995E-2</v>
+        <v>9.6931216298767886E-2</v>
       </c>
       <c r="K16" s="2">
-        <v>-3.27E-2</v>
+        <v>-4.0000000000000044E-3</v>
       </c>
       <c r="L16" s="2">
-        <v>3.7699999999999997E-2</v>
+        <v>-3.041808160000103E-3</v>
       </c>
       <c r="M16" s="2">
-        <v>0.21640000000000001</v>
+        <v>3.0660799999999929E-2</v>
       </c>
       <c r="N16" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.22454925336440401</v>
       </c>
       <c r="O16" s="2">
-        <v>8.6499999999999994E-2</v>
+        <v>8.844086955805297E-2</v>
       </c>
       <c r="P16" s="2">
-        <v>0.11119999999999999</v>
+        <v>0.1534472761844223</v>
       </c>
       <c r="Q16" s="2">
-        <v>8.6699999999999999E-2</v>
+        <v>8.8153012204149617E-2</v>
       </c>
       <c r="R16" s="2">
-        <v>7.46E-2</v>
+        <v>7.5294552309795204E-2</v>
       </c>
       <c r="S16" s="2">
-        <v>0.17899999999999999</v>
+        <v>0.1789907355690501</v>
       </c>
       <c r="T16" s="2">
-        <v>0.1026</v>
+        <v>0.1026385713853166</v>
       </c>
       <c r="U16" s="2">
-        <v>1.4999999999999999E-2</v>
+        <v>1.4977591714025349E-2</v>
       </c>
       <c r="V16" s="2">
-        <v>0.30120000000000002</v>
+        <v>0.3011668696139127</v>
       </c>
       <c r="W16" s="2">
-        <v>2.9399999999999999E-2</v>
+        <v>2.9379985875004119E-2</v>
       </c>
       <c r="X16" s="2">
-        <v>0.2051</v>
+        <v>0.2051281246826844</v>
       </c>
       <c r="Y16" s="2">
-        <v>-0.10290000000000001</v>
+        <v>-0.10290435971538731</v>
       </c>
       <c r="Z16" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.21639791486141899</v>
       </c>
       <c r="AA16" s="2">
-        <v>0.1202</v>
+        <v>0.12021853546487481</v>
       </c>
       <c r="AB16" s="2">
-        <v>-5.8599999999999999E-2</v>
+        <v>-5.861422986020437E-2</v>
       </c>
       <c r="AC16" s="2">
-        <v>0.25090000000000001</v>
+        <v>0.25087973789207202</v>
       </c>
       <c r="AD16" s="2">
-        <v>5.5899999999999998E-2</v>
+        <v>5.5915166451887321E-2</v>
       </c>
       <c r="AE16" s="2">
-        <v>0.2288</v>
+        <v>0.22876839007651761</v>
       </c>
       <c r="AF16" s="2">
-        <v>-8.8900000000000007E-2</v>
+        <v>-8.8861093780151279E-2</v>
+      </c>
+      <c r="AG16">
+        <v>5253093.3</v>
       </c>
     </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>51</v>
       </c>
@@ -2235,97 +2295,100 @@
         <v>52</v>
       </c>
       <c r="C17" s="2">
-        <v>8.0000000000000004E-4</v>
+        <v>-2.3705708333333301E-2</v>
       </c>
       <c r="D17" s="2">
-        <v>2.7799999999999998E-2</v>
+        <v>2.4300625670954371E-2</v>
       </c>
       <c r="E17" s="2">
-        <v>0.1925</v>
+        <v>2.344137605359364E-2</v>
       </c>
       <c r="F17" s="2">
-        <v>0.1925</v>
+        <v>0.14150176970463829</v>
       </c>
       <c r="G17" s="2">
-        <v>6.2300000000000001E-2</v>
+        <v>9.6726345575876893E-2</v>
       </c>
       <c r="H17" s="2">
-        <v>0.1026</v>
+        <v>0.12530952665806391</v>
       </c>
       <c r="I17" s="2">
-        <v>0.11210000000000001</v>
+        <v>0.10596760780018059</v>
       </c>
       <c r="J17" s="2">
-        <v>8.2299999999999998E-2</v>
+        <v>8.2773748212795484E-2</v>
       </c>
       <c r="K17" s="2">
-        <v>2.8999999999999998E-3</v>
+        <v>-1.129999999999998E-2</v>
       </c>
       <c r="L17" s="2">
-        <v>5.4100000000000002E-2</v>
+        <v>3.2023172983999697E-2</v>
       </c>
       <c r="M17" s="2">
-        <v>0.28149999999999997</v>
+        <v>2.9038960000000062E-2</v>
       </c>
       <c r="N17" s="2">
-        <v>0.28149999999999997</v>
+        <v>0.22217808931760799</v>
       </c>
       <c r="O17" s="2">
-        <v>0.10150000000000001</v>
+        <v>0.1285784993239765</v>
       </c>
       <c r="P17" s="2">
-        <v>0.1201</v>
+        <v>0.1515182028381199</v>
       </c>
       <c r="Q17" s="2">
-        <v>0.1145</v>
+        <v>0.10932933684393251</v>
       </c>
       <c r="R17" s="2">
-        <v>8.1799999999999998E-2</v>
+        <v>8.2549190928752791E-2</v>
       </c>
       <c r="S17" s="2">
-        <v>0.1925</v>
+        <v>0.19251440061512121</v>
       </c>
       <c r="T17" s="2">
-        <v>0.1414</v>
+        <v>0.14144707145853319</v>
       </c>
       <c r="U17" s="2">
-        <v>-0.1193</v>
+        <v>-0.119339609569489</v>
       </c>
       <c r="V17" s="2">
-        <v>0.17780000000000001</v>
+        <v>0.17776070452224821</v>
       </c>
       <c r="W17" s="2">
-        <v>0.15429999999999999</v>
+        <v>0.15429357627026061</v>
       </c>
       <c r="X17" s="2">
-        <v>0.19950000000000001</v>
+        <v>0.19951799007801679</v>
       </c>
       <c r="Y17" s="2">
-        <v>1.18E-2</v>
+        <v>1.175024958400717E-2</v>
       </c>
       <c r="Z17" s="2">
-        <v>0.28149999999999997</v>
+        <v>0.2815483740958018</v>
       </c>
       <c r="AA17" s="2">
-        <v>0.19089999999999999</v>
+        <v>0.19088023426714379</v>
       </c>
       <c r="AB17" s="2">
-        <v>-0.12429999999999999</v>
+        <v>-0.1242951408520198</v>
       </c>
       <c r="AC17" s="2">
-        <v>0.17519999999999999</v>
+        <v>0.17523622407634301</v>
       </c>
       <c r="AD17" s="2">
-        <v>0.1225</v>
+        <v>0.1225417737020502</v>
       </c>
       <c r="AE17" s="2">
-        <v>0.20200000000000001</v>
+        <v>0.2019868939492451</v>
       </c>
       <c r="AF17" s="2">
-        <v>-1.26E-2</v>
+        <v>-1.2569244036318761E-2</v>
+      </c>
+      <c r="AG17">
+        <v>28973759.07</v>
       </c>
     </row>
-    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>53</v>
       </c>
@@ -2333,97 +2396,100 @@
         <v>54</v>
       </c>
       <c r="C18" s="2">
-        <v>-7.1999999999999998E-3</v>
+        <v>8.2566551724136961E-3</v>
       </c>
       <c r="D18" s="2">
-        <v>-3.7999999999999999E-2</v>
+        <v>6.9968365460913562E-2</v>
       </c>
       <c r="E18" s="2">
-        <v>0.12379999999999999</v>
+        <v>7.7673882364492908E-2</v>
       </c>
       <c r="F18" s="2">
-        <v>0.12379999999999999</v>
+        <v>0.1408914004992097</v>
       </c>
       <c r="G18" s="2">
-        <v>4.4699999999999997E-2</v>
+        <v>9.6323739561103183E-2</v>
       </c>
       <c r="H18" s="2">
-        <v>5.4600000000000003E-2</v>
+        <v>9.6970367994610562E-2</v>
       </c>
       <c r="I18" s="2">
-        <v>5.9400000000000001E-2</v>
+        <v>6.3852103991039577E-2</v>
       </c>
       <c r="J18" s="2">
-        <v>6.1499999999999999E-2</v>
+        <v>6.7415623409172509E-2</v>
       </c>
       <c r="K18" s="2">
-        <v>4.1000000000000003E-3</v>
+        <v>1.3700000000000051E-2</v>
       </c>
       <c r="L18" s="2">
-        <v>-2.1100000000000001E-2</v>
+        <v>7.913111143400009E-2</v>
       </c>
       <c r="M18" s="2">
-        <v>0.1381</v>
+        <v>7.4724740000000178E-2</v>
       </c>
       <c r="N18" s="2">
-        <v>0.1381</v>
+        <v>0.16088398918518679</v>
       </c>
       <c r="O18" s="2">
-        <v>6.6799999999999998E-2</v>
+        <v>0.1100918047856789</v>
       </c>
       <c r="P18" s="2">
-        <v>7.2300000000000003E-2</v>
+        <v>0.1128371284909728</v>
       </c>
       <c r="Q18" s="2">
-        <v>6.9199999999999998E-2</v>
+        <v>7.3560596447728166E-2</v>
       </c>
       <c r="R18" s="2">
-        <v>7.0599999999999996E-2</v>
+        <v>7.6153486414625826E-2</v>
       </c>
       <c r="S18" s="2">
-        <v>0.12379999999999999</v>
+        <v>0.1238325144064758</v>
       </c>
       <c r="T18" s="2">
-        <v>0.1603</v>
+        <v>0.1603299067404467</v>
       </c>
       <c r="U18" s="2">
-        <v>-0.12559999999999999</v>
+        <v>-0.12561674946454729</v>
       </c>
       <c r="V18" s="2">
-        <v>4.82E-2</v>
+        <v>4.8196984917406649E-2</v>
       </c>
       <c r="W18" s="2">
-        <v>9.1600000000000001E-2</v>
+        <v>9.1570236649640702E-2</v>
       </c>
       <c r="X18" s="2">
-        <v>0.14019999999999999</v>
+        <v>0.14015252299746009</v>
       </c>
       <c r="Y18" s="2">
-        <v>-7.2099999999999997E-2</v>
+        <v>-7.2063760598472859E-2</v>
       </c>
       <c r="Z18" s="2">
-        <v>0.1381</v>
+        <v>0.13811859200861359</v>
       </c>
       <c r="AA18" s="2">
-        <v>0.15670000000000001</v>
+        <v>0.1566567055638326</v>
       </c>
       <c r="AB18" s="2">
-        <v>-7.7700000000000005E-2</v>
+        <v>-7.7705292109581325E-2</v>
       </c>
       <c r="AC18" s="2">
-        <v>0.1082</v>
+        <v>0.10817931502983601</v>
       </c>
       <c r="AD18" s="2">
-        <v>5.3800000000000001E-2</v>
+        <v>5.377222737175158E-2</v>
       </c>
       <c r="AE18" s="2">
-        <v>0.16450000000000001</v>
+        <v>0.1645435923658487</v>
       </c>
       <c r="AF18" s="2">
-        <v>-5.5500000000000001E-2</v>
+        <v>-5.5537819245731417E-2</v>
+      </c>
+      <c r="AG18">
+        <v>20320475.079999998</v>
       </c>
     </row>
-    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>55</v>
       </c>
@@ -2431,97 +2497,100 @@
         <v>33</v>
       </c>
       <c r="C19" s="2">
-        <v>-2.3300000000000001E-2</v>
+        <v>-3.1554166666666328E-3</v>
       </c>
       <c r="D19" s="2">
-        <v>2.69E-2</v>
+        <v>4.8339672149866342E-3</v>
       </c>
       <c r="E19" s="2">
-        <v>0.1706</v>
+        <v>2.8802117109006261E-2</v>
       </c>
       <c r="F19" s="2">
-        <v>0.1706</v>
+        <v>0.17157620436662491</v>
       </c>
       <c r="G19" s="2">
-        <v>0.11700000000000001</v>
+        <v>0.1022847200262036</v>
       </c>
       <c r="H19" s="2">
-        <v>0.112</v>
+        <v>0.15971397231577281</v>
       </c>
       <c r="I19" s="2">
-        <v>8.8200000000000001E-2</v>
+        <v>8.9002833803629278E-2</v>
       </c>
       <c r="J19" s="2">
-        <v>8.5599999999999996E-2</v>
+        <v>8.6420627476248457E-2</v>
       </c>
       <c r="K19" s="2">
-        <v>-3.27E-2</v>
+        <v>-4.0000000000000044E-3</v>
       </c>
       <c r="L19" s="2">
-        <v>3.7699999999999997E-2</v>
+        <v>-3.041808160000103E-3</v>
       </c>
       <c r="M19" s="2">
-        <v>0.21640000000000001</v>
+        <v>3.0660799999999929E-2</v>
       </c>
       <c r="N19" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.22454925336440401</v>
       </c>
       <c r="O19" s="2">
-        <v>8.6499999999999994E-2</v>
+        <v>8.844086955805297E-2</v>
       </c>
       <c r="P19" s="2">
-        <v>0.11119999999999999</v>
+        <v>0.1534472761844223</v>
       </c>
       <c r="Q19" s="2">
-        <v>8.6699999999999999E-2</v>
+        <v>8.8153012204149617E-2</v>
       </c>
       <c r="R19" s="2">
-        <v>8.1299999999999997E-2</v>
+        <v>8.2190923454147802E-2</v>
       </c>
       <c r="S19" s="2">
-        <v>0.1706</v>
+        <v>0.17063771874488459</v>
       </c>
       <c r="T19" s="2">
-        <v>0.1082</v>
+        <v>0.10821411542389291</v>
       </c>
       <c r="U19" s="2">
-        <v>7.4300000000000005E-2</v>
+        <v>7.4346142515499869E-2</v>
       </c>
       <c r="V19" s="2">
-        <v>0.22159999999999999</v>
+        <v>0.22162757928016791</v>
       </c>
       <c r="W19" s="2">
-        <v>-1.5E-3</v>
+        <v>-1.452798809084666E-3</v>
       </c>
       <c r="X19" s="2">
-        <v>0.1855</v>
+        <v>0.1855372953368859</v>
       </c>
       <c r="Y19" s="2">
-        <v>-9.8900000000000002E-2</v>
+        <v>-9.8920016607088379E-2</v>
       </c>
       <c r="Z19" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.21639791486141899</v>
       </c>
       <c r="AA19" s="2">
-        <v>0.1202</v>
+        <v>0.12021853546487481</v>
       </c>
       <c r="AB19" s="2">
-        <v>-5.8599999999999999E-2</v>
+        <v>-5.861422986020437E-2</v>
       </c>
       <c r="AC19" s="2">
-        <v>0.25090000000000001</v>
+        <v>0.25087973789207202</v>
       </c>
       <c r="AD19" s="2">
-        <v>5.5899999999999998E-2</v>
+        <v>5.5915166451887321E-2</v>
       </c>
       <c r="AE19" s="2">
-        <v>0.2288</v>
+        <v>0.22876839007651761</v>
       </c>
       <c r="AF19" s="2">
-        <v>-8.8900000000000007E-2</v>
+        <v>-8.8861093780151279E-2</v>
+      </c>
+      <c r="AG19">
+        <v>6349880.5800000001</v>
       </c>
     </row>
-    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>56</v>
       </c>
@@ -2529,97 +2598,100 @@
         <v>33</v>
       </c>
       <c r="C20" s="2">
-        <v>-3.9100000000000003E-2</v>
+        <v>4.8459999999999059E-3</v>
       </c>
       <c r="D20" s="2">
-        <v>6.4000000000000003E-3</v>
+        <v>-7.8954830360582484E-3</v>
       </c>
       <c r="E20" s="2">
-        <v>0.21690000000000001</v>
+        <v>3.2441382305799848E-2</v>
       </c>
       <c r="F20" s="2">
-        <v>0.21690000000000001</v>
+        <v>0.21393152861939951</v>
       </c>
       <c r="G20" s="2">
-        <v>9.8299999999999998E-2</v>
+        <v>0.11153940092618921</v>
       </c>
       <c r="H20" s="2">
-        <v>0.1125</v>
+        <v>0.13183699266832849</v>
       </c>
       <c r="I20" s="2">
-        <v>8.9599999999999999E-2</v>
+        <v>8.8114418446086917E-2</v>
       </c>
       <c r="J20" s="2">
-        <v>8.3599999999999994E-2</v>
+        <v>8.5032396039284919E-2</v>
       </c>
       <c r="K20" s="2">
-        <v>-3.27E-2</v>
+        <v>-4.0000000000000044E-3</v>
       </c>
       <c r="L20" s="2">
-        <v>3.7699999999999997E-2</v>
+        <v>-3.041808160000103E-3</v>
       </c>
       <c r="M20" s="2">
-        <v>0.21640000000000001</v>
+        <v>3.0660799999999929E-2</v>
       </c>
       <c r="N20" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.22454925336440401</v>
       </c>
       <c r="O20" s="2">
-        <v>8.6499999999999994E-2</v>
+        <v>8.844086955805297E-2</v>
       </c>
       <c r="P20" s="2">
-        <v>0.11119999999999999</v>
+        <v>0.1534472761844223</v>
       </c>
       <c r="Q20" s="2">
-        <v>8.6699999999999999E-2</v>
+        <v>8.8153012204149617E-2</v>
       </c>
       <c r="R20" s="2">
-        <v>7.46E-2</v>
+        <v>7.6009339007235388E-2</v>
       </c>
       <c r="S20" s="2">
-        <v>0.21690000000000001</v>
+        <v>0.21693517822200331</v>
       </c>
       <c r="T20" s="2">
-        <v>0.1613</v>
+        <v>0.16128355856189081</v>
       </c>
       <c r="U20" s="2">
-        <v>-6.2700000000000006E-2</v>
+        <v>-6.265463117122505E-2</v>
       </c>
       <c r="V20" s="2">
-        <v>0.2346</v>
+        <v>0.2345884019388873</v>
       </c>
       <c r="W20" s="2">
-        <v>4.19E-2</v>
+        <v>4.1925939270043289E-2</v>
       </c>
       <c r="X20" s="2">
-        <v>0.1842</v>
+        <v>0.1841829826693191</v>
       </c>
       <c r="Y20" s="2">
-        <v>-6.4699999999999994E-2</v>
+        <v>-6.4730847858231022E-2</v>
       </c>
       <c r="Z20" s="2">
-        <v>0.21640000000000001</v>
+        <v>0.21639791486141899</v>
       </c>
       <c r="AA20" s="2">
-        <v>0.1202</v>
+        <v>0.12021853546487481</v>
       </c>
       <c r="AB20" s="2">
-        <v>-5.8599999999999999E-2</v>
+        <v>-5.861422986020437E-2</v>
       </c>
       <c r="AC20" s="2">
-        <v>0.25090000000000001</v>
+        <v>0.25087973789207202</v>
       </c>
       <c r="AD20" s="2">
-        <v>5.5899999999999998E-2</v>
+        <v>5.5915166451887321E-2</v>
       </c>
       <c r="AE20" s="2">
-        <v>0.2288</v>
+        <v>0.22876839007651761</v>
       </c>
       <c r="AF20" s="2">
-        <v>-8.8900000000000007E-2</v>
+        <v>-8.8861093780151279E-2</v>
+      </c>
+      <c r="AG20">
+        <v>11712856.67</v>
       </c>
     </row>
-    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -2627,97 +2699,100 @@
         <v>35</v>
       </c>
       <c r="C21" s="2">
-        <v>-6.7999999999999996E-3</v>
+        <v>1.324039999999993E-2</v>
       </c>
       <c r="D21" s="2">
-        <v>-5.9999999999999995E-4</v>
+        <v>1.897525914572951E-2</v>
       </c>
       <c r="E21" s="2">
-        <v>4.7800000000000002E-2</v>
+        <v>2.5923738031039981E-2</v>
       </c>
       <c r="F21" s="2">
-        <v>4.7800000000000002E-2</v>
+        <v>9.3551183475714561E-2</v>
       </c>
       <c r="G21" s="2">
-        <v>-1.1999999999999999E-3</v>
+        <v>2.010687257659249E-2</v>
       </c>
       <c r="H21" s="2">
-        <v>1.3599999999999999E-2</v>
+        <v>1.0488623387680199E-2</v>
       </c>
       <c r="I21" s="2">
-        <v>2.47E-2</v>
+        <v>2.2752768678667271E-2</v>
       </c>
       <c r="J21" s="2">
-        <v>2.7E-2</v>
+        <v>2.8516004411741399E-2</v>
       </c>
       <c r="K21" s="2">
-        <v>-6.8999999999999999E-3</v>
+        <v>1.09999999999999E-2</v>
       </c>
       <c r="L21" s="2">
-        <v>-5.0000000000000001E-4</v>
+        <v>1.607238919999987E-2</v>
       </c>
       <c r="M21" s="2">
-        <v>4.2299999999999997E-2</v>
+        <v>2.313199999999993E-2</v>
       </c>
       <c r="N21" s="2">
-        <v>4.2299999999999997E-2</v>
+        <v>8.4867214211104436E-2</v>
       </c>
       <c r="O21" s="2">
-        <v>-7.1999999999999998E-3</v>
+        <v>1.6559852705851918E-2</v>
       </c>
       <c r="P21" s="2">
-        <v>7.1999999999999998E-3</v>
+        <v>9.6988969437727945E-3</v>
       </c>
       <c r="Q21" s="2">
-        <v>1.9400000000000001E-2</v>
+        <v>1.8966073465605641E-2</v>
       </c>
       <c r="R21" s="2">
-        <v>2.8899999999999999E-2</v>
+        <v>3.02405208241141E-2</v>
       </c>
       <c r="S21" s="2">
-        <v>4.7800000000000002E-2</v>
+        <v>4.7779083879743611E-2</v>
       </c>
       <c r="T21" s="2">
-        <v>7.1300000000000002E-2</v>
+        <v>7.1266059690755723E-2</v>
       </c>
       <c r="U21" s="2">
-        <v>-0.1123</v>
+        <v>-0.1122760042000059</v>
       </c>
       <c r="V21" s="2">
-        <v>-2.9499999999999998E-2</v>
+        <v>-2.948019697857374E-2</v>
       </c>
       <c r="W21" s="2">
-        <v>0.1065</v>
+        <v>0.106471440358697</v>
       </c>
       <c r="X21" s="2">
-        <v>5.9799999999999999E-2</v>
+        <v>5.9792896594321743E-2</v>
       </c>
       <c r="Y21" s="2">
-        <v>2.3400000000000001E-2</v>
+        <v>2.3394529554544349E-2</v>
       </c>
       <c r="Z21" s="2">
-        <v>4.2299999999999997E-2</v>
+        <v>4.2257028382391093E-2</v>
       </c>
       <c r="AA21" s="2">
-        <v>6.3100000000000003E-2</v>
+        <v>6.3062276236460102E-2</v>
       </c>
       <c r="AB21" s="2">
-        <v>-0.1169</v>
+        <v>-0.11689077106871799</v>
       </c>
       <c r="AC21" s="2">
-        <v>-2.5399999999999999E-2</v>
+        <v>-2.5394156876443419E-2</v>
       </c>
       <c r="AD21" s="2">
-        <v>8.6800000000000002E-2</v>
+        <v>8.6757289789715752E-2</v>
       </c>
       <c r="AE21" s="2">
-        <v>6.8699999999999997E-2</v>
+        <v>6.8712084440473165E-2</v>
       </c>
       <c r="AF21" s="2">
-        <v>1.41E-2</v>
+        <v>1.4079379818825901E-2</v>
+      </c>
+      <c r="AG21">
+        <v>14267134.48</v>
       </c>
     </row>
-    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>58</v>
       </c>
@@ -2725,97 +2800,100 @@
         <v>59</v>
       </c>
       <c r="C22" s="2">
-        <v>-7.4000000000000003E-3</v>
+        <v>-2.6336000000000141E-3</v>
       </c>
       <c r="D22" s="2">
-        <v>3.4299999999999997E-2</v>
+        <v>1.397849875872903E-2</v>
       </c>
       <c r="E22" s="2">
-        <v>0.18479999999999999</v>
+        <v>2.1534482868160069E-2</v>
       </c>
       <c r="F22" s="2">
-        <v>0.18479999999999999</v>
+        <v>0.1692093334857572</v>
       </c>
       <c r="G22" s="2">
-        <v>6.4799999999999996E-2</v>
+        <v>9.3698566827340679E-2</v>
       </c>
       <c r="H22" s="2">
-        <v>0.1195</v>
+        <v>0.12639633226276409</v>
       </c>
       <c r="I22" s="2">
-        <v>9.0399999999999994E-2</v>
+        <v>8.5653959042940819E-2</v>
       </c>
       <c r="J22" s="2">
-        <v>7.8899999999999998E-2</v>
+        <v>7.9562964955743665E-2</v>
       </c>
       <c r="K22" s="2">
-        <v>-1.2500000000000001E-2</v>
+        <v>-6.0000000000004494E-4</v>
       </c>
       <c r="L22" s="2">
-        <v>2.9899999999999999E-2</v>
+        <v>1.454091000000002E-2</v>
       </c>
       <c r="M22" s="2">
-        <v>0.1663</v>
+        <v>2.7383200000000048E-2</v>
       </c>
       <c r="N22" s="2">
-        <v>0.1663</v>
+        <v>0.16857064026149021</v>
       </c>
       <c r="O22" s="2">
-        <v>5.7099999999999998E-2</v>
+        <v>7.8351080805980189E-2</v>
       </c>
       <c r="P22" s="2">
-        <v>7.9399999999999998E-2</v>
+        <v>9.3119569427335902E-2</v>
       </c>
       <c r="Q22" s="2">
-        <v>7.4200000000000002E-2</v>
+        <v>7.20206902255216E-2</v>
       </c>
       <c r="R22" s="2">
-        <v>7.5700000000000003E-2</v>
+        <v>7.6882374514131824E-2</v>
       </c>
       <c r="S22" s="2">
-        <v>0.18479999999999999</v>
+        <v>0.1847901072070588</v>
       </c>
       <c r="T22" s="2">
-        <v>0.14130000000000001</v>
+        <v>0.14129585786912119</v>
       </c>
       <c r="U22" s="2">
-        <v>-0.1072</v>
+        <v>-0.10715189023336751</v>
       </c>
       <c r="V22" s="2">
-        <v>0.1391</v>
+        <v>0.1390876955281328</v>
       </c>
       <c r="W22" s="2">
-        <v>0.27879999999999999</v>
+        <v>0.27876690576895458</v>
       </c>
       <c r="X22" s="2">
-        <v>0.12970000000000001</v>
+        <v>0.12965554966895601</v>
       </c>
       <c r="Y22" s="2">
-        <v>-2.6599999999999999E-2</v>
+        <v>-2.6555424912946379E-2</v>
       </c>
       <c r="Z22" s="2">
-        <v>0.1663</v>
+        <v>0.1663275792250731</v>
       </c>
       <c r="AA22" s="2">
-        <v>0.124</v>
+        <v>0.1240317190194777</v>
       </c>
       <c r="AB22" s="2">
-        <v>-9.9000000000000005E-2</v>
+        <v>-9.8973580499673863E-2</v>
       </c>
       <c r="AC22" s="2">
-        <v>0.13109999999999999</v>
+        <v>0.1310961488382727</v>
       </c>
       <c r="AD22" s="2">
-        <v>9.6799999999999997E-2</v>
+        <v>9.6828978745500338E-2</v>
       </c>
       <c r="AE22" s="2">
-        <v>0.1578</v>
+        <v>0.1578400001663933</v>
       </c>
       <c r="AF22" s="2">
-        <v>-1.6400000000000001E-2</v>
+        <v>-1.6408690648921479E-2</v>
+      </c>
+      <c r="AG22">
+        <v>19726848.460000001</v>
       </c>
     </row>
-    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>60</v>
       </c>
@@ -2823,486 +2901,697 @@
         <v>37</v>
       </c>
       <c r="C23" s="2">
-        <v>6.7000000000000002E-3</v>
+        <v>-6.7880000000000162E-3</v>
       </c>
       <c r="D23" s="2">
-        <v>4.8300000000000003E-2</v>
+        <v>4.1896258212239079E-2</v>
       </c>
       <c r="E23" s="2">
-        <v>0.26719999999999999</v>
+        <v>3.4978153739199991E-2</v>
       </c>
       <c r="F23" s="2">
-        <v>0.26719999999999999</v>
+        <v>0.21055853512591319</v>
       </c>
       <c r="G23" s="2">
-        <v>0.11070000000000001</v>
+        <v>0.15860979903130759</v>
       </c>
       <c r="H23" s="2">
-        <v>0.13200000000000001</v>
+        <v>0.1456791414784904</v>
       </c>
       <c r="I23" s="2">
-        <v>0.1129</v>
+        <v>0.10452799556353611</v>
       </c>
       <c r="J23" s="2">
-        <v>0.1133</v>
+        <v>0.11463783363348901</v>
       </c>
       <c r="K23" s="2">
-        <v>4.0000000000000002E-4</v>
+        <v>-1.2499999999999961E-2</v>
       </c>
       <c r="L23" s="2">
-        <v>6.2899999999999998E-2</v>
+        <v>2.9880537499999971E-2</v>
       </c>
       <c r="M23" s="2">
-        <v>0.29430000000000001</v>
+        <v>2.9468749999999929E-2</v>
       </c>
       <c r="N23" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.2279335112320855</v>
       </c>
       <c r="O23" s="2">
-        <v>0.114</v>
+        <v>0.1406458000440951</v>
       </c>
       <c r="P23" s="2">
-        <v>0.13700000000000001</v>
+        <v>0.1663213492098834</v>
       </c>
       <c r="Q23" s="2">
-        <v>0.12770000000000001</v>
+        <v>0.12248757151155699</v>
       </c>
       <c r="R23" s="2">
-        <v>0.13350000000000001</v>
+        <v>0.13418966053852779</v>
       </c>
       <c r="S23" s="2">
-        <v>0.26719999999999999</v>
+        <v>0.26716999713421141</v>
       </c>
       <c r="T23" s="2">
-        <v>0.1724</v>
+        <v>0.17242431806507999</v>
       </c>
       <c r="U23" s="2">
-        <v>-7.7600000000000002E-2</v>
+        <v>-7.7608178432540642E-2</v>
       </c>
       <c r="V23" s="2">
-        <v>0.26850000000000002</v>
+        <v>0.2685087416826839</v>
       </c>
       <c r="W23" s="2">
-        <v>6.9500000000000006E-2</v>
+        <v>6.9484493602757436E-2</v>
       </c>
       <c r="X23" s="2">
-        <v>0.18579999999999999</v>
+        <v>0.18579928386096009</v>
       </c>
       <c r="Y23" s="2">
-        <v>-1.7299999999999999E-2</v>
+        <v>-1.734092389593855E-2</v>
       </c>
       <c r="Z23" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.29426365037508218</v>
       </c>
       <c r="AA23" s="2">
-        <v>0.2102</v>
+        <v>0.21016918258785361</v>
       </c>
       <c r="AB23" s="2">
-        <v>-0.11749999999999999</v>
+        <v>-0.1174573603921328</v>
       </c>
       <c r="AC23" s="2">
-        <v>0.21310000000000001</v>
+        <v>0.21310109733026381</v>
       </c>
       <c r="AD23" s="2">
-        <v>0.13320000000000001</v>
+        <v>0.13322710348184111</v>
       </c>
       <c r="AE23" s="2">
-        <v>0.21909999999999999</v>
+        <v>0.21910476774026419</v>
       </c>
       <c r="AF23" s="2">
-        <v>5.9999999999999995E-4</v>
+        <v>6.3113667818059938E-4</v>
+      </c>
+      <c r="AG23">
+        <v>49686620.32</v>
       </c>
     </row>
-    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="C24" s="2">
-        <v>2.7000000000000001E-3</v>
+        <v>2.3241214975864288E-3</v>
       </c>
       <c r="D24" s="2">
-        <v>8.0000000000000002E-3</v>
+        <v>6.9885816688028957E-3</v>
       </c>
       <c r="E24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>4.6536445359084411E-3</v>
       </c>
       <c r="F24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="G24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="H24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="I24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="J24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="K24" s="2">
-        <v>2.7000000000000001E-3</v>
+        <v>2.3241214975864288E-3</v>
       </c>
       <c r="L24" s="2">
-        <v>8.0000000000000002E-3</v>
+        <v>6.9885816688028957E-3</v>
       </c>
       <c r="M24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>4.6536445359084411E-3</v>
       </c>
       <c r="N24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="O24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="P24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="Q24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="R24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="S24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="T24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="U24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="V24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="W24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="X24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="Y24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="Z24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="AA24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="AB24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="AC24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="AD24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="AE24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
       </c>
       <c r="AF24" s="2">
-        <v>3.2300000000000002E-2</v>
+        <v>2.824873600000001E-2</v>
+      </c>
+      <c r="AG24">
+        <v>33829548.840000004</v>
       </c>
     </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B25" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="C25" s="2">
-        <v>2.5999999999999999E-3</v>
+        <v>2.2554219815378311E-3</v>
       </c>
       <c r="D25" s="2">
-        <v>7.7999999999999996E-3</v>
+        <v>6.7815382027280879E-3</v>
       </c>
       <c r="E25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>4.5159308913906848E-3</v>
       </c>
       <c r="F25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="G25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="H25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="I25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="J25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="K25" s="2">
-        <v>2.5999999999999999E-3</v>
+        <v>2.2554219815378311E-3</v>
       </c>
       <c r="L25" s="2">
-        <v>7.7999999999999996E-3</v>
+        <v>6.7815382027280879E-3</v>
       </c>
       <c r="M25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>4.5159308913906848E-3</v>
       </c>
       <c r="N25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="O25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="P25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="Q25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="R25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="S25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="T25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="U25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="V25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="W25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="X25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="Y25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="Z25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="AA25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="AB25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="AC25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="AD25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="AE25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
       </c>
       <c r="AF25" s="2">
-        <v>3.1699999999999999E-2</v>
+        <v>2.7403337999999999E-2</v>
+      </c>
+      <c r="AG25">
+        <v>120284577.84</v>
       </c>
     </row>
-    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="C26" s="2">
-        <v>4.0000000000000002E-4</v>
+        <v>1.0799999999999921E-2</v>
       </c>
       <c r="D26" s="2">
-        <v>6.2899999999999998E-2</v>
+        <v>1.393457166399981E-2</v>
       </c>
       <c r="E26" s="2">
-        <v>0.29430000000000001</v>
+        <v>1.352915999999982E-2</v>
       </c>
       <c r="F26" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.20892102861296771</v>
       </c>
       <c r="G26" s="2">
-        <v>0.114</v>
+        <v>0.13472815943675381</v>
       </c>
       <c r="H26" s="2">
-        <v>0.13700000000000001</v>
+        <v>0.16268706625506771</v>
       </c>
       <c r="I26" s="2">
-        <v>0.12770000000000001</v>
+        <v>0.1207373590525465</v>
       </c>
       <c r="J26" s="2">
-        <v>9.3299999999999994E-2</v>
+        <v>9.3237092723982951E-2</v>
       </c>
       <c r="K26" s="2">
-        <v>4.0000000000000002E-4</v>
+        <v>-1.2499999999999961E-2</v>
       </c>
       <c r="L26" s="2">
-        <v>6.2899999999999998E-2</v>
+        <v>2.9880537499999971E-2</v>
       </c>
       <c r="M26" s="2">
-        <v>0.29430000000000001</v>
+        <v>2.9468749999999929E-2</v>
       </c>
       <c r="N26" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.2279335112320855</v>
       </c>
       <c r="O26" s="2">
-        <v>0.114</v>
+        <v>0.1406458000440951</v>
       </c>
       <c r="P26" s="2">
-        <v>0.13700000000000001</v>
+        <v>0.1663213492098834</v>
       </c>
       <c r="Q26" s="2">
-        <v>0.12770000000000001</v>
+        <v>0.12248757151155699</v>
       </c>
       <c r="R26" s="2">
-        <v>9.3299999999999994E-2</v>
+        <v>9.4006958248271877E-2</v>
       </c>
       <c r="S26" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.29426365037508218</v>
       </c>
       <c r="T26" s="2">
-        <v>0.2102</v>
+        <v>0.21016918258785361</v>
       </c>
       <c r="U26" s="2">
-        <v>-0.11749999999999999</v>
+        <v>-0.1174573603921328</v>
       </c>
       <c r="V26" s="2">
-        <v>0.21310000000000001</v>
+        <v>0.21310109733026381</v>
       </c>
       <c r="W26" s="2">
-        <v>0.13320000000000001</v>
+        <v>0.13322710348184111</v>
       </c>
       <c r="X26" s="2">
-        <v>0.21909999999999999</v>
+        <v>0.21910476774026419</v>
       </c>
       <c r="Y26" s="2">
-        <v>5.9999999999999995E-4</v>
+        <v>6.3113667818059938E-4</v>
       </c>
       <c r="Z26" s="2">
-        <v>0.29430000000000001</v>
+        <v>0.29426365037508218</v>
       </c>
       <c r="AA26" s="2">
-        <v>0.2102</v>
+        <v>0.21016918258785361</v>
       </c>
       <c r="AB26" s="2">
-        <v>-0.11749999999999999</v>
+        <v>-0.1174573603921328</v>
       </c>
       <c r="AC26" s="2">
-        <v>0.21310000000000001</v>
+        <v>0.21310109733026381</v>
       </c>
       <c r="AD26" s="2">
-        <v>0.13320000000000001</v>
+        <v>0.13322710348184111</v>
       </c>
       <c r="AE26" s="2">
-        <v>0.21909999999999999</v>
+        <v>0.21910476774026419</v>
       </c>
       <c r="AF26" s="2">
-        <v>5.9999999999999995E-4</v>
+        <v>6.3113667818059938E-4</v>
+      </c>
+      <c r="AG26">
+        <v>566421.62</v>
       </c>
     </row>
-    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>61</v>
       </c>
       <c r="B27" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="C27" s="3">
-        <v>-1.11E-2</v>
+        <v>1.2999999999999901E-2</v>
       </c>
       <c r="D27" s="3">
-        <v>1.24E-2</v>
+        <v>2.8001699340000071E-2</v>
       </c>
       <c r="E27" s="3">
-        <v>0.12479999999999999</v>
+        <v>3.9540599999999808E-2</v>
       </c>
       <c r="F27" s="3">
-        <v>0.12479999999999999</v>
+        <v>0.170802098022663</v>
       </c>
       <c r="G27" s="3">
-        <v>4.6199999999999998E-2</v>
+        <v>6.4271526647182275E-2</v>
       </c>
       <c r="H27" s="3">
-        <v>5.3999999999999999E-2</v>
+        <v>6.4043482811291463E-2</v>
       </c>
       <c r="I27" s="3">
-        <v>5.5599999999999997E-2</v>
+        <v>5.2621985378944032E-2</v>
       </c>
       <c r="J27" s="3">
-        <v>6.3200000000000006E-2</v>
+        <v>6.4674870986276112E-2</v>
       </c>
       <c r="K27" s="3">
-        <v>-1.11E-2</v>
+        <v>1.2999999999999901E-2</v>
       </c>
       <c r="L27" s="3">
-        <v>1.24E-2</v>
+        <v>2.8001699340000071E-2</v>
       </c>
       <c r="M27" s="3">
-        <v>0.12479999999999999</v>
+        <v>3.9540599999999808E-2</v>
       </c>
       <c r="N27" s="3">
-        <v>0.12479999999999999</v>
+        <v>0.170802098022663</v>
       </c>
       <c r="O27" s="3">
-        <v>4.6199999999999998E-2</v>
+        <v>6.4271526647182275E-2</v>
       </c>
       <c r="P27" s="3">
-        <v>5.3999999999999999E-2</v>
+        <v>6.4043482811291463E-2</v>
       </c>
       <c r="Q27" s="3">
-        <v>5.5599999999999997E-2</v>
+        <v>5.2621985378944032E-2</v>
       </c>
       <c r="R27" s="3">
-        <v>6.3200000000000006E-2</v>
+        <v>6.4674870986276112E-2</v>
       </c>
       <c r="S27" s="3">
-        <v>0.12479999999999999</v>
+        <v>0.124788964358634</v>
       </c>
       <c r="T27" s="3">
-        <v>5.4100000000000002E-2</v>
+        <v>5.4098630863060437E-2</v>
       </c>
       <c r="U27" s="3">
-        <v>-3.4200000000000001E-2</v>
+        <v>-3.4202652847085679E-2</v>
       </c>
       <c r="V27" s="3">
-        <v>0.14560000000000001</v>
+        <v>0.1455653061407236</v>
       </c>
       <c r="W27" s="3">
-        <v>-8.3000000000000001E-3</v>
+        <v>-8.3092281574879134E-3</v>
       </c>
       <c r="X27" s="3">
-        <v>0.1159</v>
+        <v>0.115914764648821</v>
       </c>
       <c r="Y27" s="3">
-        <v>2.01E-2</v>
+        <v>2.0091365915979601E-2</v>
       </c>
       <c r="Z27" s="3">
-        <v>0.12479999999999999</v>
+        <v>0.124788964358634</v>
       </c>
       <c r="AA27" s="3">
-        <v>5.4100000000000002E-2</v>
+        <v>5.4098630863060437E-2</v>
       </c>
       <c r="AB27" s="3">
-        <v>-3.4200000000000001E-2</v>
+        <v>-3.4202652847085679E-2</v>
       </c>
       <c r="AC27" s="3">
-        <v>0.14560000000000001</v>
+        <v>0.1455653061407236</v>
       </c>
       <c r="AD27" s="3">
-        <v>-8.3000000000000001E-3</v>
+        <v>-8.3092281574879134E-3</v>
       </c>
       <c r="AE27" s="3">
-        <v>0.1159</v>
+        <v>0.115914764648821</v>
       </c>
       <c r="AF27" s="3">
-        <v>2.01E-2</v>
+        <v>2.0091365915979601E-2</v>
+      </c>
+      <c r="AG27">
+        <v>8496363.8900000006</v>
+      </c>
+    </row>
+    <row r="28" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="3">
+        <v>-8.0935342777976871E-5</v>
+      </c>
+      <c r="D28" s="3">
+        <v>1.041737660673658E-2</v>
+      </c>
+      <c r="E28" s="3">
+        <v>5.7255080201208397E-3</v>
+      </c>
+      <c r="F28" s="3">
+        <v>7.0769775235454357E-2</v>
+      </c>
+      <c r="G28" s="3">
+        <v>6.6794600907987611E-2</v>
+      </c>
+      <c r="H28" s="3">
+        <v>5.5185384468519061E-2</v>
+      </c>
+      <c r="I28" s="3">
+        <v>4.4717103155460507E-2</v>
+      </c>
+      <c r="J28" s="3">
+        <v>5.006258815824971E-2</v>
+      </c>
+      <c r="K28" s="3">
+        <v>-8.0935342777976871E-5</v>
+      </c>
+      <c r="L28" s="3">
+        <v>1.041737660673658E-2</v>
+      </c>
+      <c r="M28" s="3">
+        <v>5.7255080201208397E-3</v>
+      </c>
+      <c r="N28" s="3">
+        <v>7.0769775235454357E-2</v>
+      </c>
+      <c r="O28" s="3">
+        <v>6.6794600907987611E-2</v>
+      </c>
+      <c r="P28" s="3">
+        <v>5.5185384468519061E-2</v>
+      </c>
+      <c r="Q28" s="3">
+        <v>4.4717103155460507E-2</v>
+      </c>
+      <c r="R28" s="3">
+        <v>5.006258815824971E-2</v>
+      </c>
+      <c r="S28" s="3">
+        <v>8.0714217637701147E-2</v>
+      </c>
+      <c r="T28" s="3">
+        <v>0.1259456759958231</v>
+      </c>
+      <c r="U28" s="3">
+        <v>-9.3833560932529148E-3</v>
+      </c>
+      <c r="V28" s="3">
+        <v>5.1052418973622782E-2</v>
+      </c>
+      <c r="W28" s="3">
+        <v>1.828699955803148E-2</v>
+      </c>
+      <c r="X28" s="3">
+        <v>7.7349186294291661E-2</v>
+      </c>
+      <c r="Y28" s="3">
+        <v>-4.6128794597813938E-3</v>
+      </c>
+      <c r="Z28" s="3">
+        <v>8.0714217637701147E-2</v>
+      </c>
+      <c r="AA28" s="3">
+        <v>0.1259456759958231</v>
+      </c>
+      <c r="AB28" s="3">
+        <v>-9.3833560932529148E-3</v>
+      </c>
+      <c r="AC28" s="3">
+        <v>5.1052418973622782E-2</v>
+      </c>
+      <c r="AD28" s="3">
+        <v>1.828699955803148E-2</v>
+      </c>
+      <c r="AE28" s="3">
+        <v>7.7349186294291661E-2</v>
+      </c>
+      <c r="AF28" s="3">
+        <v>-4.6128794597813938E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>74</v>
+      </c>
+      <c r="B29" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="3">
+        <v>1.727040000000013E-3</v>
+      </c>
+      <c r="D29" s="3">
+        <v>5.3565368763467847E-2</v>
+      </c>
+      <c r="E29" s="3">
+        <v>6.5419740194345488E-2</v>
+      </c>
+      <c r="F29" s="3">
+        <v>9.2357935205118924E-2</v>
+      </c>
+      <c r="G29" s="3">
+        <v>8.6845983915933234E-2</v>
+      </c>
+      <c r="H29" s="3">
+        <v>9.1369689936083631E-2</v>
+      </c>
+      <c r="I29" s="3">
+        <v>6.2527939087650086E-2</v>
+      </c>
+      <c r="J29" s="3">
+        <v>7.5988108111384678E-2</v>
+      </c>
+      <c r="K29" s="3">
+        <v>1.3700000000000051E-2</v>
+      </c>
+      <c r="L29" s="3">
+        <v>7.913111143400009E-2</v>
+      </c>
+      <c r="M29" s="3">
+        <v>7.4724740000000178E-2</v>
+      </c>
+      <c r="N29" s="3">
+        <v>0.16088398918518679</v>
+      </c>
+      <c r="O29" s="3">
+        <v>0.1100918047856789</v>
+      </c>
+      <c r="P29" s="3">
+        <v>0.1128371284909728</v>
+      </c>
+      <c r="Q29" s="3">
+        <v>7.3560596447728166E-2</v>
+      </c>
+      <c r="R29" s="3">
+        <v>7.5666529305396413E-2</v>
+      </c>
+      <c r="S29" s="3">
+        <v>9.2049378719037733E-2</v>
+      </c>
+      <c r="T29" s="3">
+        <v>0.1898117381043074</v>
+      </c>
+      <c r="U29" s="3">
+        <v>-0.1603738713607461</v>
+      </c>
+      <c r="V29" s="3">
+        <v>0.16507135840840581</v>
+      </c>
+      <c r="W29" s="3">
+        <v>5.4079106591117247E-2</v>
+      </c>
+      <c r="X29" s="3">
+        <v>0.15845914942998779</v>
+      </c>
+      <c r="Y29" s="3">
+        <v>-6.0255804356564857E-2</v>
+      </c>
+      <c r="Z29" s="3">
+        <v>0.13811859200861359</v>
+      </c>
+      <c r="AA29" s="3">
+        <v>0.1566567055638326</v>
+      </c>
+      <c r="AB29" s="3">
+        <v>-7.7705292109581325E-2</v>
+      </c>
+      <c r="AC29" s="3">
+        <v>0.10817931502983601</v>
+      </c>
+      <c r="AD29" s="3">
+        <v>5.377222737175158E-2</v>
+      </c>
+      <c r="AE29" s="3">
+        <v>0.1645435923658487</v>
+      </c>
+      <c r="AF29" s="3">
+        <v>-5.5537819245731417E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>